<commit_message>
docs(skills): replace product-specific terms with generic ones
- numbered image skill: describe the spec list mode by an item number and
  a layer node id instead of named CSV columns
- spec template: permission columns become 管理者, 編集者, 閲覧者

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/skills/screen-detail-spec-excel/assets/screen-detail-spec-template.xlsx
+++ b/skills/screen-detail-spec-excel/assets/screen-detail-spec-template.xlsx
@@ -2656,17 +2656,17 @@
       </c>
       <c r="J86" s="2" t="inlineStr">
         <is>
-          <t>project_admin</t>
+          <t>管理者</t>
         </is>
       </c>
       <c r="K86" s="2" t="inlineStr">
         <is>
-          <t>member</t>
+          <t>編集者</t>
         </is>
       </c>
       <c r="L86" s="2" t="inlineStr">
         <is>
-          <t>viewer</t>
+          <t>閲覧者</t>
         </is>
       </c>
       <c r="M86" s="13" t="n"/>

</xml_diff>

<commit_message>
feat(skills): ask before writing and simplify the spec template
- Add research, question and quality references: source ranking and an
  evidence map, one consolidated question round before writing, and a
  checklist run before delivery
- Template: drop the permission table and the source column; the message
  table keeps one Japanese column 表示メッセージ
- README: describe the question round

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/skills/screen-detail-spec-excel/assets/screen-detail-spec-template.xlsx
+++ b/skills/screen-detail-spec-excel/assets/screen-detail-spec-template.xlsx
@@ -695,7 +695,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:V145"/>
+  <dimension ref="B1:U132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -718,8 +718,7 @@
     <col width="30" customWidth="1" min="18" max="18"/>
     <col width="18" customWidth="1" min="19" max="19"/>
     <col width="18" customWidth="1" min="20" max="20"/>
-    <col width="28" customWidth="1" min="21" max="21"/>
-    <col width="24" customWidth="1" min="22" max="22"/>
+    <col width="40" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -746,7 +745,6 @@
       <c r="S1" s="6" t="n"/>
       <c r="T1" s="6" t="n"/>
       <c r="U1" s="6" t="n"/>
-      <c r="V1" s="6" t="n"/>
     </row>
     <row r="2">
       <c r="B2" s="7" t="inlineStr">
@@ -784,7 +782,6 @@
       <c r="S2" s="8" t="n"/>
       <c r="T2" s="8" t="n"/>
       <c r="U2" s="8" t="n"/>
-      <c r="V2" s="8" t="n"/>
     </row>
     <row r="3" ht="45" customHeight="1">
       <c r="B3" s="7" t="inlineStr">
@@ -810,7 +807,6 @@
       <c r="S3" s="8" t="n"/>
       <c r="T3" s="8" t="n"/>
       <c r="U3" s="8" t="n"/>
-      <c r="V3" s="8" t="n"/>
     </row>
     <row r="4">
       <c r="B4" s="7" t="inlineStr">
@@ -872,7 +868,6 @@
       <c r="S6" s="11" t="n"/>
       <c r="T6" s="11" t="n"/>
       <c r="U6" s="11" t="n"/>
-      <c r="V6" s="11" t="n"/>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="12" t="inlineStr">
@@ -968,11 +963,6 @@
       <c r="U7" s="2" t="inlineStr">
         <is>
           <t>データベース備考</t>
-        </is>
-      </c>
-      <c r="V7" s="2" t="inlineStr">
-        <is>
-          <t>出典</t>
         </is>
       </c>
     </row>
@@ -996,7 +986,6 @@
       <c r="S8" s="3" t="n"/>
       <c r="T8" s="3" t="n"/>
       <c r="U8" s="3" t="n"/>
-      <c r="V8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="B9" s="8" t="n"/>
@@ -1018,7 +1007,6 @@
       <c r="S9" s="3" t="n"/>
       <c r="T9" s="3" t="n"/>
       <c r="U9" s="3" t="n"/>
-      <c r="V9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="B10" s="8" t="n"/>
@@ -1040,7 +1028,6 @@
       <c r="S10" s="3" t="n"/>
       <c r="T10" s="3" t="n"/>
       <c r="U10" s="3" t="n"/>
-      <c r="V10" s="3" t="n"/>
     </row>
     <row r="11">
       <c r="B11" s="8" t="n"/>
@@ -1062,7 +1049,6 @@
       <c r="S11" s="3" t="n"/>
       <c r="T11" s="3" t="n"/>
       <c r="U11" s="3" t="n"/>
-      <c r="V11" s="3" t="n"/>
     </row>
     <row r="12">
       <c r="B12" s="8" t="n"/>
@@ -1084,7 +1070,6 @@
       <c r="S12" s="3" t="n"/>
       <c r="T12" s="3" t="n"/>
       <c r="U12" s="3" t="n"/>
-      <c r="V12" s="3" t="n"/>
     </row>
     <row r="13">
       <c r="B13" s="8" t="n"/>
@@ -1106,7 +1091,6 @@
       <c r="S13" s="3" t="n"/>
       <c r="T13" s="3" t="n"/>
       <c r="U13" s="3" t="n"/>
-      <c r="V13" s="3" t="n"/>
     </row>
     <row r="14">
       <c r="B14" s="8" t="n"/>
@@ -1128,7 +1112,6 @@
       <c r="S14" s="3" t="n"/>
       <c r="T14" s="3" t="n"/>
       <c r="U14" s="3" t="n"/>
-      <c r="V14" s="3" t="n"/>
     </row>
     <row r="15">
       <c r="B15" s="8" t="n"/>
@@ -1150,7 +1133,6 @@
       <c r="S15" s="3" t="n"/>
       <c r="T15" s="3" t="n"/>
       <c r="U15" s="3" t="n"/>
-      <c r="V15" s="3" t="n"/>
     </row>
     <row r="16">
       <c r="B16" s="8" t="n"/>
@@ -1172,7 +1154,6 @@
       <c r="S16" s="3" t="n"/>
       <c r="T16" s="3" t="n"/>
       <c r="U16" s="3" t="n"/>
-      <c r="V16" s="3" t="n"/>
     </row>
     <row r="17">
       <c r="B17" s="8" t="n"/>
@@ -1194,7 +1175,6 @@
       <c r="S17" s="3" t="n"/>
       <c r="T17" s="3" t="n"/>
       <c r="U17" s="3" t="n"/>
-      <c r="V17" s="3" t="n"/>
     </row>
     <row r="18">
       <c r="B18" s="8" t="n"/>
@@ -1216,7 +1196,6 @@
       <c r="S18" s="3" t="n"/>
       <c r="T18" s="3" t="n"/>
       <c r="U18" s="3" t="n"/>
-      <c r="V18" s="3" t="n"/>
     </row>
     <row r="19">
       <c r="B19" s="8" t="n"/>
@@ -1238,7 +1217,6 @@
       <c r="S19" s="3" t="n"/>
       <c r="T19" s="3" t="n"/>
       <c r="U19" s="3" t="n"/>
-      <c r="V19" s="3" t="n"/>
     </row>
     <row r="20">
       <c r="B20" s="8" t="n"/>
@@ -1260,7 +1238,6 @@
       <c r="S20" s="3" t="n"/>
       <c r="T20" s="3" t="n"/>
       <c r="U20" s="3" t="n"/>
-      <c r="V20" s="3" t="n"/>
     </row>
     <row r="21">
       <c r="B21" s="8" t="n"/>
@@ -1282,7 +1259,6 @@
       <c r="S21" s="3" t="n"/>
       <c r="T21" s="3" t="n"/>
       <c r="U21" s="3" t="n"/>
-      <c r="V21" s="3" t="n"/>
     </row>
     <row r="22">
       <c r="B22" s="8" t="n"/>
@@ -1304,7 +1280,6 @@
       <c r="S22" s="3" t="n"/>
       <c r="T22" s="3" t="n"/>
       <c r="U22" s="3" t="n"/>
-      <c r="V22" s="3" t="n"/>
     </row>
     <row r="23">
       <c r="B23" s="8" t="n"/>
@@ -1326,7 +1301,6 @@
       <c r="S23" s="3" t="n"/>
       <c r="T23" s="3" t="n"/>
       <c r="U23" s="3" t="n"/>
-      <c r="V23" s="3" t="n"/>
     </row>
     <row r="24">
       <c r="B24" s="8" t="n"/>
@@ -1348,7 +1322,6 @@
       <c r="S24" s="3" t="n"/>
       <c r="T24" s="3" t="n"/>
       <c r="U24" s="3" t="n"/>
-      <c r="V24" s="3" t="n"/>
     </row>
     <row r="25">
       <c r="B25" s="8" t="n"/>
@@ -1370,7 +1343,6 @@
       <c r="S25" s="3" t="n"/>
       <c r="T25" s="3" t="n"/>
       <c r="U25" s="3" t="n"/>
-      <c r="V25" s="3" t="n"/>
     </row>
     <row r="26">
       <c r="B26" s="8" t="n"/>
@@ -1392,7 +1364,6 @@
       <c r="S26" s="3" t="n"/>
       <c r="T26" s="3" t="n"/>
       <c r="U26" s="3" t="n"/>
-      <c r="V26" s="3" t="n"/>
     </row>
     <row r="27">
       <c r="B27" s="8" t="n"/>
@@ -1414,7 +1385,6 @@
       <c r="S27" s="3" t="n"/>
       <c r="T27" s="3" t="n"/>
       <c r="U27" s="3" t="n"/>
-      <c r="V27" s="3" t="n"/>
     </row>
     <row r="28">
       <c r="B28" s="8" t="n"/>
@@ -1436,7 +1406,6 @@
       <c r="S28" s="3" t="n"/>
       <c r="T28" s="3" t="n"/>
       <c r="U28" s="3" t="n"/>
-      <c r="V28" s="3" t="n"/>
     </row>
     <row r="29">
       <c r="B29" s="8" t="n"/>
@@ -1458,7 +1427,6 @@
       <c r="S29" s="3" t="n"/>
       <c r="T29" s="3" t="n"/>
       <c r="U29" s="3" t="n"/>
-      <c r="V29" s="3" t="n"/>
     </row>
     <row r="30">
       <c r="B30" s="8" t="n"/>
@@ -1480,7 +1448,6 @@
       <c r="S30" s="3" t="n"/>
       <c r="T30" s="3" t="n"/>
       <c r="U30" s="3" t="n"/>
-      <c r="V30" s="3" t="n"/>
     </row>
     <row r="31">
       <c r="B31" s="8" t="n"/>
@@ -1502,7 +1469,6 @@
       <c r="S31" s="3" t="n"/>
       <c r="T31" s="3" t="n"/>
       <c r="U31" s="3" t="n"/>
-      <c r="V31" s="3" t="n"/>
     </row>
     <row r="32">
       <c r="B32" s="8" t="n"/>
@@ -1524,7 +1490,6 @@
       <c r="S32" s="3" t="n"/>
       <c r="T32" s="3" t="n"/>
       <c r="U32" s="3" t="n"/>
-      <c r="V32" s="3" t="n"/>
     </row>
     <row r="33">
       <c r="B33" s="8" t="n"/>
@@ -1546,7 +1511,6 @@
       <c r="S33" s="3" t="n"/>
       <c r="T33" s="3" t="n"/>
       <c r="U33" s="3" t="n"/>
-      <c r="V33" s="3" t="n"/>
     </row>
     <row r="34">
       <c r="B34" s="8" t="n"/>
@@ -1568,7 +1532,6 @@
       <c r="S34" s="3" t="n"/>
       <c r="T34" s="3" t="n"/>
       <c r="U34" s="3" t="n"/>
-      <c r="V34" s="3" t="n"/>
     </row>
     <row r="35">
       <c r="B35" s="8" t="n"/>
@@ -1590,7 +1553,6 @@
       <c r="S35" s="3" t="n"/>
       <c r="T35" s="3" t="n"/>
       <c r="U35" s="3" t="n"/>
-      <c r="V35" s="3" t="n"/>
     </row>
     <row r="36">
       <c r="B36" s="8" t="n"/>
@@ -1612,7 +1574,6 @@
       <c r="S36" s="3" t="n"/>
       <c r="T36" s="3" t="n"/>
       <c r="U36" s="3" t="n"/>
-      <c r="V36" s="3" t="n"/>
     </row>
     <row r="37">
       <c r="B37" s="8" t="n"/>
@@ -1634,7 +1595,6 @@
       <c r="S37" s="3" t="n"/>
       <c r="T37" s="3" t="n"/>
       <c r="U37" s="3" t="n"/>
-      <c r="V37" s="3" t="n"/>
     </row>
     <row r="38">
       <c r="B38" s="8" t="n"/>
@@ -1656,7 +1616,6 @@
       <c r="S38" s="3" t="n"/>
       <c r="T38" s="3" t="n"/>
       <c r="U38" s="3" t="n"/>
-      <c r="V38" s="3" t="n"/>
     </row>
     <row r="39">
       <c r="B39" s="8" t="n"/>
@@ -1678,7 +1637,6 @@
       <c r="S39" s="3" t="n"/>
       <c r="T39" s="3" t="n"/>
       <c r="U39" s="3" t="n"/>
-      <c r="V39" s="3" t="n"/>
     </row>
     <row r="40">
       <c r="B40" s="8" t="n"/>
@@ -1700,7 +1658,6 @@
       <c r="S40" s="3" t="n"/>
       <c r="T40" s="3" t="n"/>
       <c r="U40" s="3" t="n"/>
-      <c r="V40" s="3" t="n"/>
     </row>
     <row r="41">
       <c r="B41" s="8" t="n"/>
@@ -1722,7 +1679,6 @@
       <c r="S41" s="3" t="n"/>
       <c r="T41" s="3" t="n"/>
       <c r="U41" s="3" t="n"/>
-      <c r="V41" s="3" t="n"/>
     </row>
     <row r="42">
       <c r="B42" s="8" t="n"/>
@@ -1744,7 +1700,6 @@
       <c r="S42" s="3" t="n"/>
       <c r="T42" s="3" t="n"/>
       <c r="U42" s="3" t="n"/>
-      <c r="V42" s="3" t="n"/>
     </row>
     <row r="43">
       <c r="B43" s="8" t="n"/>
@@ -1766,7 +1721,6 @@
       <c r="S43" s="3" t="n"/>
       <c r="T43" s="3" t="n"/>
       <c r="U43" s="3" t="n"/>
-      <c r="V43" s="3" t="n"/>
     </row>
     <row r="44">
       <c r="B44" s="8" t="n"/>
@@ -1788,7 +1742,6 @@
       <c r="S44" s="3" t="n"/>
       <c r="T44" s="3" t="n"/>
       <c r="U44" s="3" t="n"/>
-      <c r="V44" s="3" t="n"/>
     </row>
     <row r="45">
       <c r="B45" s="8" t="n"/>
@@ -1810,7 +1763,6 @@
       <c r="S45" s="3" t="n"/>
       <c r="T45" s="3" t="n"/>
       <c r="U45" s="3" t="n"/>
-      <c r="V45" s="3" t="n"/>
     </row>
     <row r="46">
       <c r="B46" s="8" t="n"/>
@@ -1832,7 +1784,6 @@
       <c r="S46" s="3" t="n"/>
       <c r="T46" s="3" t="n"/>
       <c r="U46" s="3" t="n"/>
-      <c r="V46" s="3" t="n"/>
     </row>
     <row r="47">
       <c r="B47" s="8" t="n"/>
@@ -1854,7 +1805,6 @@
       <c r="S47" s="3" t="n"/>
       <c r="T47" s="3" t="n"/>
       <c r="U47" s="3" t="n"/>
-      <c r="V47" s="3" t="n"/>
     </row>
     <row r="49" ht="22" customHeight="1">
       <c r="D49" s="10" t="inlineStr">
@@ -1879,7 +1829,6 @@
       <c r="S49" s="11" t="n"/>
       <c r="T49" s="11" t="n"/>
       <c r="U49" s="11" t="n"/>
-      <c r="V49" s="11" t="n"/>
     </row>
     <row r="50" ht="30" customHeight="1">
       <c r="D50" s="2" t="inlineStr">
@@ -1909,14 +1858,9 @@
       <c r="P50" s="13" t="n"/>
       <c r="Q50" s="13" t="n"/>
       <c r="R50" s="13" t="n"/>
-      <c r="S50" s="2" t="inlineStr">
-        <is>
-          <t>出典</t>
-        </is>
-      </c>
+      <c r="S50" s="13" t="n"/>
       <c r="T50" s="13" t="n"/>
       <c r="U50" s="13" t="n"/>
-      <c r="V50" s="13" t="n"/>
     </row>
     <row r="51">
       <c r="D51" s="3" t="n"/>
@@ -1934,10 +1878,9 @@
       <c r="P51" s="8" t="n"/>
       <c r="Q51" s="8" t="n"/>
       <c r="R51" s="8" t="n"/>
-      <c r="S51" s="3" t="n"/>
+      <c r="S51" s="8" t="n"/>
       <c r="T51" s="8" t="n"/>
       <c r="U51" s="8" t="n"/>
-      <c r="V51" s="8" t="n"/>
     </row>
     <row r="52">
       <c r="D52" s="3" t="n"/>
@@ -1955,10 +1898,9 @@
       <c r="P52" s="8" t="n"/>
       <c r="Q52" s="8" t="n"/>
       <c r="R52" s="8" t="n"/>
-      <c r="S52" s="3" t="n"/>
+      <c r="S52" s="8" t="n"/>
       <c r="T52" s="8" t="n"/>
       <c r="U52" s="8" t="n"/>
-      <c r="V52" s="8" t="n"/>
     </row>
     <row r="53">
       <c r="D53" s="3" t="n"/>
@@ -1976,10 +1918,9 @@
       <c r="P53" s="8" t="n"/>
       <c r="Q53" s="8" t="n"/>
       <c r="R53" s="8" t="n"/>
-      <c r="S53" s="3" t="n"/>
+      <c r="S53" s="8" t="n"/>
       <c r="T53" s="8" t="n"/>
       <c r="U53" s="8" t="n"/>
-      <c r="V53" s="8" t="n"/>
     </row>
     <row r="54">
       <c r="D54" s="3" t="n"/>
@@ -1997,10 +1938,9 @@
       <c r="P54" s="8" t="n"/>
       <c r="Q54" s="8" t="n"/>
       <c r="R54" s="8" t="n"/>
-      <c r="S54" s="3" t="n"/>
+      <c r="S54" s="8" t="n"/>
       <c r="T54" s="8" t="n"/>
       <c r="U54" s="8" t="n"/>
-      <c r="V54" s="8" t="n"/>
     </row>
     <row r="55">
       <c r="D55" s="3" t="n"/>
@@ -2018,10 +1958,9 @@
       <c r="P55" s="8" t="n"/>
       <c r="Q55" s="8" t="n"/>
       <c r="R55" s="8" t="n"/>
-      <c r="S55" s="3" t="n"/>
+      <c r="S55" s="8" t="n"/>
       <c r="T55" s="8" t="n"/>
       <c r="U55" s="8" t="n"/>
-      <c r="V55" s="8" t="n"/>
     </row>
     <row r="56">
       <c r="D56" s="3" t="n"/>
@@ -2039,10 +1978,9 @@
       <c r="P56" s="8" t="n"/>
       <c r="Q56" s="8" t="n"/>
       <c r="R56" s="8" t="n"/>
-      <c r="S56" s="3" t="n"/>
+      <c r="S56" s="8" t="n"/>
       <c r="T56" s="8" t="n"/>
       <c r="U56" s="8" t="n"/>
-      <c r="V56" s="8" t="n"/>
     </row>
     <row r="57">
       <c r="D57" s="3" t="n"/>
@@ -2060,10 +1998,9 @@
       <c r="P57" s="8" t="n"/>
       <c r="Q57" s="8" t="n"/>
       <c r="R57" s="8" t="n"/>
-      <c r="S57" s="3" t="n"/>
+      <c r="S57" s="8" t="n"/>
       <c r="T57" s="8" t="n"/>
       <c r="U57" s="8" t="n"/>
-      <c r="V57" s="8" t="n"/>
     </row>
     <row r="58">
       <c r="D58" s="3" t="n"/>
@@ -2081,10 +2018,9 @@
       <c r="P58" s="8" t="n"/>
       <c r="Q58" s="8" t="n"/>
       <c r="R58" s="8" t="n"/>
-      <c r="S58" s="3" t="n"/>
+      <c r="S58" s="8" t="n"/>
       <c r="T58" s="8" t="n"/>
       <c r="U58" s="8" t="n"/>
-      <c r="V58" s="8" t="n"/>
     </row>
     <row r="59">
       <c r="D59" s="3" t="n"/>
@@ -2102,10 +2038,9 @@
       <c r="P59" s="8" t="n"/>
       <c r="Q59" s="8" t="n"/>
       <c r="R59" s="8" t="n"/>
-      <c r="S59" s="3" t="n"/>
+      <c r="S59" s="8" t="n"/>
       <c r="T59" s="8" t="n"/>
       <c r="U59" s="8" t="n"/>
-      <c r="V59" s="8" t="n"/>
     </row>
     <row r="60">
       <c r="D60" s="3" t="n"/>
@@ -2123,10 +2058,9 @@
       <c r="P60" s="8" t="n"/>
       <c r="Q60" s="8" t="n"/>
       <c r="R60" s="8" t="n"/>
-      <c r="S60" s="3" t="n"/>
+      <c r="S60" s="8" t="n"/>
       <c r="T60" s="8" t="n"/>
       <c r="U60" s="8" t="n"/>
-      <c r="V60" s="8" t="n"/>
     </row>
     <row r="61">
       <c r="D61" s="3" t="n"/>
@@ -2144,10 +2078,9 @@
       <c r="P61" s="8" t="n"/>
       <c r="Q61" s="8" t="n"/>
       <c r="R61" s="8" t="n"/>
-      <c r="S61" s="3" t="n"/>
+      <c r="S61" s="8" t="n"/>
       <c r="T61" s="8" t="n"/>
       <c r="U61" s="8" t="n"/>
-      <c r="V61" s="8" t="n"/>
     </row>
     <row r="62">
       <c r="D62" s="3" t="n"/>
@@ -2165,10 +2098,9 @@
       <c r="P62" s="8" t="n"/>
       <c r="Q62" s="8" t="n"/>
       <c r="R62" s="8" t="n"/>
-      <c r="S62" s="3" t="n"/>
+      <c r="S62" s="8" t="n"/>
       <c r="T62" s="8" t="n"/>
       <c r="U62" s="8" t="n"/>
-      <c r="V62" s="8" t="n"/>
     </row>
     <row r="63">
       <c r="D63" s="3" t="n"/>
@@ -2186,10 +2118,9 @@
       <c r="P63" s="8" t="n"/>
       <c r="Q63" s="8" t="n"/>
       <c r="R63" s="8" t="n"/>
-      <c r="S63" s="3" t="n"/>
+      <c r="S63" s="8" t="n"/>
       <c r="T63" s="8" t="n"/>
       <c r="U63" s="8" t="n"/>
-      <c r="V63" s="8" t="n"/>
     </row>
     <row r="64">
       <c r="D64" s="3" t="n"/>
@@ -2207,10 +2138,9 @@
       <c r="P64" s="8" t="n"/>
       <c r="Q64" s="8" t="n"/>
       <c r="R64" s="8" t="n"/>
-      <c r="S64" s="3" t="n"/>
+      <c r="S64" s="8" t="n"/>
       <c r="T64" s="8" t="n"/>
       <c r="U64" s="8" t="n"/>
-      <c r="V64" s="8" t="n"/>
     </row>
     <row r="65">
       <c r="D65" s="3" t="n"/>
@@ -2228,10 +2158,9 @@
       <c r="P65" s="8" t="n"/>
       <c r="Q65" s="8" t="n"/>
       <c r="R65" s="8" t="n"/>
-      <c r="S65" s="3" t="n"/>
+      <c r="S65" s="8" t="n"/>
       <c r="T65" s="8" t="n"/>
       <c r="U65" s="8" t="n"/>
-      <c r="V65" s="8" t="n"/>
     </row>
     <row r="67" ht="22" customHeight="1">
       <c r="D67" s="10" t="inlineStr">
@@ -2256,7 +2185,6 @@
       <c r="S67" s="11" t="n"/>
       <c r="T67" s="11" t="n"/>
       <c r="U67" s="11" t="n"/>
-      <c r="V67" s="11" t="n"/>
     </row>
     <row r="68" ht="30" customHeight="1">
       <c r="D68" s="2" t="inlineStr">
@@ -2290,14 +2218,9 @@
       <c r="P68" s="13" t="n"/>
       <c r="Q68" s="13" t="n"/>
       <c r="R68" s="13" t="n"/>
-      <c r="S68" s="2" t="inlineStr">
-        <is>
-          <t>出典</t>
-        </is>
-      </c>
+      <c r="S68" s="13" t="n"/>
       <c r="T68" s="13" t="n"/>
       <c r="U68" s="13" t="n"/>
-      <c r="V68" s="13" t="n"/>
     </row>
     <row r="69">
       <c r="D69" s="3" t="n"/>
@@ -2315,10 +2238,9 @@
       <c r="P69" s="8" t="n"/>
       <c r="Q69" s="8" t="n"/>
       <c r="R69" s="8" t="n"/>
-      <c r="S69" s="3" t="n"/>
+      <c r="S69" s="8" t="n"/>
       <c r="T69" s="8" t="n"/>
       <c r="U69" s="8" t="n"/>
-      <c r="V69" s="8" t="n"/>
     </row>
     <row r="70">
       <c r="D70" s="3" t="n"/>
@@ -2336,10 +2258,9 @@
       <c r="P70" s="8" t="n"/>
       <c r="Q70" s="8" t="n"/>
       <c r="R70" s="8" t="n"/>
-      <c r="S70" s="3" t="n"/>
+      <c r="S70" s="8" t="n"/>
       <c r="T70" s="8" t="n"/>
       <c r="U70" s="8" t="n"/>
-      <c r="V70" s="8" t="n"/>
     </row>
     <row r="71">
       <c r="D71" s="3" t="n"/>
@@ -2357,10 +2278,9 @@
       <c r="P71" s="8" t="n"/>
       <c r="Q71" s="8" t="n"/>
       <c r="R71" s="8" t="n"/>
-      <c r="S71" s="3" t="n"/>
+      <c r="S71" s="8" t="n"/>
       <c r="T71" s="8" t="n"/>
       <c r="U71" s="8" t="n"/>
-      <c r="V71" s="8" t="n"/>
     </row>
     <row r="72">
       <c r="D72" s="3" t="n"/>
@@ -2378,10 +2298,9 @@
       <c r="P72" s="8" t="n"/>
       <c r="Q72" s="8" t="n"/>
       <c r="R72" s="8" t="n"/>
-      <c r="S72" s="3" t="n"/>
+      <c r="S72" s="8" t="n"/>
       <c r="T72" s="8" t="n"/>
       <c r="U72" s="8" t="n"/>
-      <c r="V72" s="8" t="n"/>
     </row>
     <row r="73">
       <c r="D73" s="3" t="n"/>
@@ -2399,10 +2318,9 @@
       <c r="P73" s="8" t="n"/>
       <c r="Q73" s="8" t="n"/>
       <c r="R73" s="8" t="n"/>
-      <c r="S73" s="3" t="n"/>
+      <c r="S73" s="8" t="n"/>
       <c r="T73" s="8" t="n"/>
       <c r="U73" s="8" t="n"/>
-      <c r="V73" s="8" t="n"/>
     </row>
     <row r="74">
       <c r="D74" s="3" t="n"/>
@@ -2420,10 +2338,9 @@
       <c r="P74" s="8" t="n"/>
       <c r="Q74" s="8" t="n"/>
       <c r="R74" s="8" t="n"/>
-      <c r="S74" s="3" t="n"/>
+      <c r="S74" s="8" t="n"/>
       <c r="T74" s="8" t="n"/>
       <c r="U74" s="8" t="n"/>
-      <c r="V74" s="8" t="n"/>
     </row>
     <row r="75">
       <c r="D75" s="3" t="n"/>
@@ -2441,10 +2358,9 @@
       <c r="P75" s="8" t="n"/>
       <c r="Q75" s="8" t="n"/>
       <c r="R75" s="8" t="n"/>
-      <c r="S75" s="3" t="n"/>
+      <c r="S75" s="8" t="n"/>
       <c r="T75" s="8" t="n"/>
       <c r="U75" s="8" t="n"/>
-      <c r="V75" s="8" t="n"/>
     </row>
     <row r="76">
       <c r="D76" s="3" t="n"/>
@@ -2462,10 +2378,9 @@
       <c r="P76" s="8" t="n"/>
       <c r="Q76" s="8" t="n"/>
       <c r="R76" s="8" t="n"/>
-      <c r="S76" s="3" t="n"/>
+      <c r="S76" s="8" t="n"/>
       <c r="T76" s="8" t="n"/>
       <c r="U76" s="8" t="n"/>
-      <c r="V76" s="8" t="n"/>
     </row>
     <row r="77">
       <c r="D77" s="3" t="n"/>
@@ -2483,10 +2398,9 @@
       <c r="P77" s="8" t="n"/>
       <c r="Q77" s="8" t="n"/>
       <c r="R77" s="8" t="n"/>
-      <c r="S77" s="3" t="n"/>
+      <c r="S77" s="8" t="n"/>
       <c r="T77" s="8" t="n"/>
       <c r="U77" s="8" t="n"/>
-      <c r="V77" s="8" t="n"/>
     </row>
     <row r="78">
       <c r="D78" s="3" t="n"/>
@@ -2504,10 +2418,9 @@
       <c r="P78" s="8" t="n"/>
       <c r="Q78" s="8" t="n"/>
       <c r="R78" s="8" t="n"/>
-      <c r="S78" s="3" t="n"/>
+      <c r="S78" s="8" t="n"/>
       <c r="T78" s="8" t="n"/>
       <c r="U78" s="8" t="n"/>
-      <c r="V78" s="8" t="n"/>
     </row>
     <row r="79">
       <c r="D79" s="3" t="n"/>
@@ -2525,10 +2438,9 @@
       <c r="P79" s="8" t="n"/>
       <c r="Q79" s="8" t="n"/>
       <c r="R79" s="8" t="n"/>
-      <c r="S79" s="3" t="n"/>
+      <c r="S79" s="8" t="n"/>
       <c r="T79" s="8" t="n"/>
       <c r="U79" s="8" t="n"/>
-      <c r="V79" s="8" t="n"/>
     </row>
     <row r="80">
       <c r="D80" s="3" t="n"/>
@@ -2546,10 +2458,9 @@
       <c r="P80" s="8" t="n"/>
       <c r="Q80" s="8" t="n"/>
       <c r="R80" s="8" t="n"/>
-      <c r="S80" s="3" t="n"/>
+      <c r="S80" s="8" t="n"/>
       <c r="T80" s="8" t="n"/>
       <c r="U80" s="8" t="n"/>
-      <c r="V80" s="8" t="n"/>
     </row>
     <row r="81">
       <c r="D81" s="3" t="n"/>
@@ -2567,10 +2478,9 @@
       <c r="P81" s="8" t="n"/>
       <c r="Q81" s="8" t="n"/>
       <c r="R81" s="8" t="n"/>
-      <c r="S81" s="3" t="n"/>
+      <c r="S81" s="8" t="n"/>
       <c r="T81" s="8" t="n"/>
       <c r="U81" s="8" t="n"/>
-      <c r="V81" s="8" t="n"/>
     </row>
     <row r="82">
       <c r="D82" s="3" t="n"/>
@@ -2588,10 +2498,9 @@
       <c r="P82" s="8" t="n"/>
       <c r="Q82" s="8" t="n"/>
       <c r="R82" s="8" t="n"/>
-      <c r="S82" s="3" t="n"/>
+      <c r="S82" s="8" t="n"/>
       <c r="T82" s="8" t="n"/>
       <c r="U82" s="8" t="n"/>
-      <c r="V82" s="8" t="n"/>
     </row>
     <row r="83">
       <c r="D83" s="3" t="n"/>
@@ -2609,15 +2518,14 @@
       <c r="P83" s="8" t="n"/>
       <c r="Q83" s="8" t="n"/>
       <c r="R83" s="8" t="n"/>
-      <c r="S83" s="3" t="n"/>
+      <c r="S83" s="8" t="n"/>
       <c r="T83" s="8" t="n"/>
       <c r="U83" s="8" t="n"/>
-      <c r="V83" s="8" t="n"/>
     </row>
     <row r="85" ht="22" customHeight="1">
       <c r="D85" s="10" t="inlineStr">
         <is>
-          <t>権限</t>
+          <t>エラー処理</t>
         </is>
       </c>
       <c r="E85" s="11" t="n"/>
@@ -2637,267 +2545,259 @@
       <c r="S85" s="11" t="n"/>
       <c r="T85" s="11" t="n"/>
       <c r="U85" s="11" t="n"/>
-      <c r="V85" s="11" t="n"/>
     </row>
     <row r="86" ht="30" customHeight="1">
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>操作</t>
-        </is>
-      </c>
-      <c r="E86" s="13" t="n"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>対象項目No</t>
+        </is>
+      </c>
       <c r="F86" s="13" t="n"/>
-      <c r="G86" s="13" t="n"/>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>エラーケース</t>
+        </is>
+      </c>
       <c r="H86" s="13" t="n"/>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>対象項目No</t>
-        </is>
-      </c>
-      <c r="J86" s="2" t="inlineStr">
-        <is>
-          <t>管理者</t>
-        </is>
-      </c>
-      <c r="K86" s="2" t="inlineStr">
-        <is>
-          <t>編集者</t>
-        </is>
-      </c>
+          <t>発生条件</t>
+        </is>
+      </c>
+      <c r="J86" s="13" t="n"/>
+      <c r="K86" s="13" t="n"/>
       <c r="L86" s="2" t="inlineStr">
         <is>
-          <t>閲覧者</t>
+          <t>システムの動作</t>
         </is>
       </c>
       <c r="M86" s="13" t="n"/>
       <c r="N86" s="13" t="n"/>
       <c r="O86" s="13" t="n"/>
       <c r="P86" s="13" t="n"/>
-      <c r="Q86" s="2" t="inlineStr">
+      <c r="Q86" s="13" t="n"/>
+      <c r="R86" s="13" t="n"/>
+      <c r="S86" s="2" t="inlineStr">
+        <is>
+          <t>メッセージID</t>
+        </is>
+      </c>
+      <c r="T86" s="2" t="inlineStr">
         <is>
           <t>備考</t>
         </is>
       </c>
-      <c r="R86" s="13" t="n"/>
-      <c r="S86" s="13" t="n"/>
-      <c r="T86" s="13" t="n"/>
       <c r="U86" s="13" t="n"/>
-      <c r="V86" s="13" t="n"/>
     </row>
     <row r="87">
       <c r="D87" s="3" t="n"/>
-      <c r="E87" s="8" t="n"/>
+      <c r="E87" s="3" t="n"/>
       <c r="F87" s="8" t="n"/>
-      <c r="G87" s="8" t="n"/>
+      <c r="G87" s="3" t="n"/>
       <c r="H87" s="8" t="n"/>
       <c r="I87" s="3" t="n"/>
-      <c r="J87" s="3" t="n"/>
-      <c r="K87" s="3" t="n"/>
+      <c r="J87" s="8" t="n"/>
+      <c r="K87" s="8" t="n"/>
       <c r="L87" s="3" t="n"/>
       <c r="M87" s="8" t="n"/>
       <c r="N87" s="8" t="n"/>
       <c r="O87" s="8" t="n"/>
       <c r="P87" s="8" t="n"/>
-      <c r="Q87" s="3" t="n"/>
+      <c r="Q87" s="8" t="n"/>
       <c r="R87" s="8" t="n"/>
-      <c r="S87" s="8" t="n"/>
-      <c r="T87" s="8" t="n"/>
+      <c r="S87" s="3" t="n"/>
+      <c r="T87" s="3" t="n"/>
       <c r="U87" s="8" t="n"/>
-      <c r="V87" s="8" t="n"/>
     </row>
     <row r="88">
       <c r="D88" s="3" t="n"/>
-      <c r="E88" s="8" t="n"/>
+      <c r="E88" s="3" t="n"/>
       <c r="F88" s="8" t="n"/>
-      <c r="G88" s="8" t="n"/>
+      <c r="G88" s="3" t="n"/>
       <c r="H88" s="8" t="n"/>
       <c r="I88" s="3" t="n"/>
-      <c r="J88" s="3" t="n"/>
-      <c r="K88" s="3" t="n"/>
+      <c r="J88" s="8" t="n"/>
+      <c r="K88" s="8" t="n"/>
       <c r="L88" s="3" t="n"/>
       <c r="M88" s="8" t="n"/>
       <c r="N88" s="8" t="n"/>
       <c r="O88" s="8" t="n"/>
       <c r="P88" s="8" t="n"/>
-      <c r="Q88" s="3" t="n"/>
+      <c r="Q88" s="8" t="n"/>
       <c r="R88" s="8" t="n"/>
-      <c r="S88" s="8" t="n"/>
-      <c r="T88" s="8" t="n"/>
+      <c r="S88" s="3" t="n"/>
+      <c r="T88" s="3" t="n"/>
       <c r="U88" s="8" t="n"/>
-      <c r="V88" s="8" t="n"/>
     </row>
     <row r="89">
       <c r="D89" s="3" t="n"/>
-      <c r="E89" s="8" t="n"/>
+      <c r="E89" s="3" t="n"/>
       <c r="F89" s="8" t="n"/>
-      <c r="G89" s="8" t="n"/>
+      <c r="G89" s="3" t="n"/>
       <c r="H89" s="8" t="n"/>
       <c r="I89" s="3" t="n"/>
-      <c r="J89" s="3" t="n"/>
-      <c r="K89" s="3" t="n"/>
+      <c r="J89" s="8" t="n"/>
+      <c r="K89" s="8" t="n"/>
       <c r="L89" s="3" t="n"/>
       <c r="M89" s="8" t="n"/>
       <c r="N89" s="8" t="n"/>
       <c r="O89" s="8" t="n"/>
       <c r="P89" s="8" t="n"/>
-      <c r="Q89" s="3" t="n"/>
+      <c r="Q89" s="8" t="n"/>
       <c r="R89" s="8" t="n"/>
-      <c r="S89" s="8" t="n"/>
-      <c r="T89" s="8" t="n"/>
+      <c r="S89" s="3" t="n"/>
+      <c r="T89" s="3" t="n"/>
       <c r="U89" s="8" t="n"/>
-      <c r="V89" s="8" t="n"/>
     </row>
     <row r="90">
       <c r="D90" s="3" t="n"/>
-      <c r="E90" s="8" t="n"/>
+      <c r="E90" s="3" t="n"/>
       <c r="F90" s="8" t="n"/>
-      <c r="G90" s="8" t="n"/>
+      <c r="G90" s="3" t="n"/>
       <c r="H90" s="8" t="n"/>
       <c r="I90" s="3" t="n"/>
-      <c r="J90" s="3" t="n"/>
-      <c r="K90" s="3" t="n"/>
+      <c r="J90" s="8" t="n"/>
+      <c r="K90" s="8" t="n"/>
       <c r="L90" s="3" t="n"/>
       <c r="M90" s="8" t="n"/>
       <c r="N90" s="8" t="n"/>
       <c r="O90" s="8" t="n"/>
       <c r="P90" s="8" t="n"/>
-      <c r="Q90" s="3" t="n"/>
+      <c r="Q90" s="8" t="n"/>
       <c r="R90" s="8" t="n"/>
-      <c r="S90" s="8" t="n"/>
-      <c r="T90" s="8" t="n"/>
+      <c r="S90" s="3" t="n"/>
+      <c r="T90" s="3" t="n"/>
       <c r="U90" s="8" t="n"/>
-      <c r="V90" s="8" t="n"/>
     </row>
     <row r="91">
       <c r="D91" s="3" t="n"/>
-      <c r="E91" s="8" t="n"/>
+      <c r="E91" s="3" t="n"/>
       <c r="F91" s="8" t="n"/>
-      <c r="G91" s="8" t="n"/>
+      <c r="G91" s="3" t="n"/>
       <c r="H91" s="8" t="n"/>
       <c r="I91" s="3" t="n"/>
-      <c r="J91" s="3" t="n"/>
-      <c r="K91" s="3" t="n"/>
+      <c r="J91" s="8" t="n"/>
+      <c r="K91" s="8" t="n"/>
       <c r="L91" s="3" t="n"/>
       <c r="M91" s="8" t="n"/>
       <c r="N91" s="8" t="n"/>
       <c r="O91" s="8" t="n"/>
       <c r="P91" s="8" t="n"/>
-      <c r="Q91" s="3" t="n"/>
+      <c r="Q91" s="8" t="n"/>
       <c r="R91" s="8" t="n"/>
-      <c r="S91" s="8" t="n"/>
-      <c r="T91" s="8" t="n"/>
+      <c r="S91" s="3" t="n"/>
+      <c r="T91" s="3" t="n"/>
       <c r="U91" s="8" t="n"/>
-      <c r="V91" s="8" t="n"/>
     </row>
     <row r="92">
       <c r="D92" s="3" t="n"/>
-      <c r="E92" s="8" t="n"/>
+      <c r="E92" s="3" t="n"/>
       <c r="F92" s="8" t="n"/>
-      <c r="G92" s="8" t="n"/>
+      <c r="G92" s="3" t="n"/>
       <c r="H92" s="8" t="n"/>
       <c r="I92" s="3" t="n"/>
-      <c r="J92" s="3" t="n"/>
-      <c r="K92" s="3" t="n"/>
+      <c r="J92" s="8" t="n"/>
+      <c r="K92" s="8" t="n"/>
       <c r="L92" s="3" t="n"/>
       <c r="M92" s="8" t="n"/>
       <c r="N92" s="8" t="n"/>
       <c r="O92" s="8" t="n"/>
       <c r="P92" s="8" t="n"/>
-      <c r="Q92" s="3" t="n"/>
+      <c r="Q92" s="8" t="n"/>
       <c r="R92" s="8" t="n"/>
-      <c r="S92" s="8" t="n"/>
-      <c r="T92" s="8" t="n"/>
+      <c r="S92" s="3" t="n"/>
+      <c r="T92" s="3" t="n"/>
       <c r="U92" s="8" t="n"/>
-      <c r="V92" s="8" t="n"/>
     </row>
     <row r="93">
       <c r="D93" s="3" t="n"/>
-      <c r="E93" s="8" t="n"/>
+      <c r="E93" s="3" t="n"/>
       <c r="F93" s="8" t="n"/>
-      <c r="G93" s="8" t="n"/>
+      <c r="G93" s="3" t="n"/>
       <c r="H93" s="8" t="n"/>
       <c r="I93" s="3" t="n"/>
-      <c r="J93" s="3" t="n"/>
-      <c r="K93" s="3" t="n"/>
+      <c r="J93" s="8" t="n"/>
+      <c r="K93" s="8" t="n"/>
       <c r="L93" s="3" t="n"/>
       <c r="M93" s="8" t="n"/>
       <c r="N93" s="8" t="n"/>
       <c r="O93" s="8" t="n"/>
       <c r="P93" s="8" t="n"/>
-      <c r="Q93" s="3" t="n"/>
+      <c r="Q93" s="8" t="n"/>
       <c r="R93" s="8" t="n"/>
-      <c r="S93" s="8" t="n"/>
-      <c r="T93" s="8" t="n"/>
+      <c r="S93" s="3" t="n"/>
+      <c r="T93" s="3" t="n"/>
       <c r="U93" s="8" t="n"/>
-      <c r="V93" s="8" t="n"/>
     </row>
     <row r="94">
       <c r="D94" s="3" t="n"/>
-      <c r="E94" s="8" t="n"/>
+      <c r="E94" s="3" t="n"/>
       <c r="F94" s="8" t="n"/>
-      <c r="G94" s="8" t="n"/>
+      <c r="G94" s="3" t="n"/>
       <c r="H94" s="8" t="n"/>
       <c r="I94" s="3" t="n"/>
-      <c r="J94" s="3" t="n"/>
-      <c r="K94" s="3" t="n"/>
+      <c r="J94" s="8" t="n"/>
+      <c r="K94" s="8" t="n"/>
       <c r="L94" s="3" t="n"/>
       <c r="M94" s="8" t="n"/>
       <c r="N94" s="8" t="n"/>
       <c r="O94" s="8" t="n"/>
       <c r="P94" s="8" t="n"/>
-      <c r="Q94" s="3" t="n"/>
+      <c r="Q94" s="8" t="n"/>
       <c r="R94" s="8" t="n"/>
-      <c r="S94" s="8" t="n"/>
-      <c r="T94" s="8" t="n"/>
+      <c r="S94" s="3" t="n"/>
+      <c r="T94" s="3" t="n"/>
       <c r="U94" s="8" t="n"/>
-      <c r="V94" s="8" t="n"/>
     </row>
     <row r="95">
       <c r="D95" s="3" t="n"/>
-      <c r="E95" s="8" t="n"/>
+      <c r="E95" s="3" t="n"/>
       <c r="F95" s="8" t="n"/>
-      <c r="G95" s="8" t="n"/>
+      <c r="G95" s="3" t="n"/>
       <c r="H95" s="8" t="n"/>
       <c r="I95" s="3" t="n"/>
-      <c r="J95" s="3" t="n"/>
-      <c r="K95" s="3" t="n"/>
+      <c r="J95" s="8" t="n"/>
+      <c r="K95" s="8" t="n"/>
       <c r="L95" s="3" t="n"/>
       <c r="M95" s="8" t="n"/>
       <c r="N95" s="8" t="n"/>
       <c r="O95" s="8" t="n"/>
       <c r="P95" s="8" t="n"/>
-      <c r="Q95" s="3" t="n"/>
+      <c r="Q95" s="8" t="n"/>
       <c r="R95" s="8" t="n"/>
-      <c r="S95" s="8" t="n"/>
-      <c r="T95" s="8" t="n"/>
+      <c r="S95" s="3" t="n"/>
+      <c r="T95" s="3" t="n"/>
       <c r="U95" s="8" t="n"/>
-      <c r="V95" s="8" t="n"/>
     </row>
     <row r="96">
       <c r="D96" s="3" t="n"/>
-      <c r="E96" s="8" t="n"/>
+      <c r="E96" s="3" t="n"/>
       <c r="F96" s="8" t="n"/>
-      <c r="G96" s="8" t="n"/>
+      <c r="G96" s="3" t="n"/>
       <c r="H96" s="8" t="n"/>
       <c r="I96" s="3" t="n"/>
-      <c r="J96" s="3" t="n"/>
-      <c r="K96" s="3" t="n"/>
+      <c r="J96" s="8" t="n"/>
+      <c r="K96" s="8" t="n"/>
       <c r="L96" s="3" t="n"/>
       <c r="M96" s="8" t="n"/>
       <c r="N96" s="8" t="n"/>
       <c r="O96" s="8" t="n"/>
       <c r="P96" s="8" t="n"/>
-      <c r="Q96" s="3" t="n"/>
+      <c r="Q96" s="8" t="n"/>
       <c r="R96" s="8" t="n"/>
-      <c r="S96" s="8" t="n"/>
-      <c r="T96" s="8" t="n"/>
+      <c r="S96" s="3" t="n"/>
+      <c r="T96" s="3" t="n"/>
       <c r="U96" s="8" t="n"/>
-      <c r="V96" s="8" t="n"/>
     </row>
     <row r="98" ht="22" customHeight="1">
       <c r="D98" s="10" t="inlineStr">
         <is>
-          <t>エラー処理</t>
+          <t>メッセージ一覧</t>
         </is>
       </c>
       <c r="E98" s="11" t="n"/>
@@ -2917,340 +2817,306 @@
       <c r="S98" s="11" t="n"/>
       <c r="T98" s="11" t="n"/>
       <c r="U98" s="11" t="n"/>
-      <c r="V98" s="11" t="n"/>
     </row>
     <row r="99" ht="30" customHeight="1">
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E99" s="2" t="inlineStr">
-        <is>
-          <t>対象項目No</t>
-        </is>
-      </c>
+          <t>メッセージID</t>
+        </is>
+      </c>
+      <c r="E99" s="13" t="n"/>
       <c r="F99" s="13" t="n"/>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>エラーケース</t>
-        </is>
-      </c>
-      <c r="H99" s="13" t="n"/>
-      <c r="I99" s="2" t="inlineStr">
-        <is>
-          <t>発生条件</t>
-        </is>
-      </c>
+          <t>種別</t>
+        </is>
+      </c>
+      <c r="H99" s="2" t="inlineStr">
+        <is>
+          <t>表示メッセージ</t>
+        </is>
+      </c>
+      <c r="I99" s="13" t="n"/>
       <c r="J99" s="13" t="n"/>
       <c r="K99" s="13" t="n"/>
-      <c r="L99" s="2" t="inlineStr">
-        <is>
-          <t>システムの動作</t>
-        </is>
-      </c>
+      <c r="L99" s="13" t="n"/>
       <c r="M99" s="13" t="n"/>
       <c r="N99" s="13" t="n"/>
       <c r="O99" s="13" t="n"/>
       <c r="P99" s="13" t="n"/>
       <c r="Q99" s="13" t="n"/>
-      <c r="R99" s="13" t="n"/>
+      <c r="R99" s="2" t="inlineStr">
+        <is>
+          <t>表示方法</t>
+        </is>
+      </c>
       <c r="S99" s="2" t="inlineStr">
         <is>
-          <t>メッセージID</t>
-        </is>
-      </c>
-      <c r="T99" s="2" t="inlineStr">
-        <is>
           <t>備考</t>
         </is>
       </c>
+      <c r="T99" s="13" t="n"/>
       <c r="U99" s="13" t="n"/>
-      <c r="V99" s="13" t="n"/>
     </row>
     <row r="100">
       <c r="D100" s="3" t="n"/>
-      <c r="E100" s="3" t="n"/>
+      <c r="E100" s="8" t="n"/>
       <c r="F100" s="8" t="n"/>
       <c r="G100" s="3" t="n"/>
-      <c r="H100" s="8" t="n"/>
-      <c r="I100" s="3" t="n"/>
+      <c r="H100" s="3" t="n"/>
+      <c r="I100" s="8" t="n"/>
       <c r="J100" s="8" t="n"/>
       <c r="K100" s="8" t="n"/>
-      <c r="L100" s="3" t="n"/>
+      <c r="L100" s="8" t="n"/>
       <c r="M100" s="8" t="n"/>
       <c r="N100" s="8" t="n"/>
       <c r="O100" s="8" t="n"/>
       <c r="P100" s="8" t="n"/>
       <c r="Q100" s="8" t="n"/>
-      <c r="R100" s="8" t="n"/>
+      <c r="R100" s="3" t="n"/>
       <c r="S100" s="3" t="n"/>
-      <c r="T100" s="3" t="n"/>
+      <c r="T100" s="8" t="n"/>
       <c r="U100" s="8" t="n"/>
-      <c r="V100" s="8" t="n"/>
     </row>
     <row r="101">
       <c r="D101" s="3" t="n"/>
-      <c r="E101" s="3" t="n"/>
+      <c r="E101" s="8" t="n"/>
       <c r="F101" s="8" t="n"/>
       <c r="G101" s="3" t="n"/>
-      <c r="H101" s="8" t="n"/>
-      <c r="I101" s="3" t="n"/>
+      <c r="H101" s="3" t="n"/>
+      <c r="I101" s="8" t="n"/>
       <c r="J101" s="8" t="n"/>
       <c r="K101" s="8" t="n"/>
-      <c r="L101" s="3" t="n"/>
+      <c r="L101" s="8" t="n"/>
       <c r="M101" s="8" t="n"/>
       <c r="N101" s="8" t="n"/>
       <c r="O101" s="8" t="n"/>
       <c r="P101" s="8" t="n"/>
       <c r="Q101" s="8" t="n"/>
-      <c r="R101" s="8" t="n"/>
+      <c r="R101" s="3" t="n"/>
       <c r="S101" s="3" t="n"/>
-      <c r="T101" s="3" t="n"/>
+      <c r="T101" s="8" t="n"/>
       <c r="U101" s="8" t="n"/>
-      <c r="V101" s="8" t="n"/>
     </row>
     <row r="102">
       <c r="D102" s="3" t="n"/>
-      <c r="E102" s="3" t="n"/>
+      <c r="E102" s="8" t="n"/>
       <c r="F102" s="8" t="n"/>
       <c r="G102" s="3" t="n"/>
-      <c r="H102" s="8" t="n"/>
-      <c r="I102" s="3" t="n"/>
+      <c r="H102" s="3" t="n"/>
+      <c r="I102" s="8" t="n"/>
       <c r="J102" s="8" t="n"/>
       <c r="K102" s="8" t="n"/>
-      <c r="L102" s="3" t="n"/>
+      <c r="L102" s="8" t="n"/>
       <c r="M102" s="8" t="n"/>
       <c r="N102" s="8" t="n"/>
       <c r="O102" s="8" t="n"/>
       <c r="P102" s="8" t="n"/>
       <c r="Q102" s="8" t="n"/>
-      <c r="R102" s="8" t="n"/>
+      <c r="R102" s="3" t="n"/>
       <c r="S102" s="3" t="n"/>
-      <c r="T102" s="3" t="n"/>
+      <c r="T102" s="8" t="n"/>
       <c r="U102" s="8" t="n"/>
-      <c r="V102" s="8" t="n"/>
     </row>
     <row r="103">
       <c r="D103" s="3" t="n"/>
-      <c r="E103" s="3" t="n"/>
+      <c r="E103" s="8" t="n"/>
       <c r="F103" s="8" t="n"/>
       <c r="G103" s="3" t="n"/>
-      <c r="H103" s="8" t="n"/>
-      <c r="I103" s="3" t="n"/>
+      <c r="H103" s="3" t="n"/>
+      <c r="I103" s="8" t="n"/>
       <c r="J103" s="8" t="n"/>
       <c r="K103" s="8" t="n"/>
-      <c r="L103" s="3" t="n"/>
+      <c r="L103" s="8" t="n"/>
       <c r="M103" s="8" t="n"/>
       <c r="N103" s="8" t="n"/>
       <c r="O103" s="8" t="n"/>
       <c r="P103" s="8" t="n"/>
       <c r="Q103" s="8" t="n"/>
-      <c r="R103" s="8" t="n"/>
+      <c r="R103" s="3" t="n"/>
       <c r="S103" s="3" t="n"/>
-      <c r="T103" s="3" t="n"/>
+      <c r="T103" s="8" t="n"/>
       <c r="U103" s="8" t="n"/>
-      <c r="V103" s="8" t="n"/>
     </row>
     <row r="104">
       <c r="D104" s="3" t="n"/>
-      <c r="E104" s="3" t="n"/>
+      <c r="E104" s="8" t="n"/>
       <c r="F104" s="8" t="n"/>
       <c r="G104" s="3" t="n"/>
-      <c r="H104" s="8" t="n"/>
-      <c r="I104" s="3" t="n"/>
+      <c r="H104" s="3" t="n"/>
+      <c r="I104" s="8" t="n"/>
       <c r="J104" s="8" t="n"/>
       <c r="K104" s="8" t="n"/>
-      <c r="L104" s="3" t="n"/>
+      <c r="L104" s="8" t="n"/>
       <c r="M104" s="8" t="n"/>
       <c r="N104" s="8" t="n"/>
       <c r="O104" s="8" t="n"/>
       <c r="P104" s="8" t="n"/>
       <c r="Q104" s="8" t="n"/>
-      <c r="R104" s="8" t="n"/>
+      <c r="R104" s="3" t="n"/>
       <c r="S104" s="3" t="n"/>
-      <c r="T104" s="3" t="n"/>
+      <c r="T104" s="8" t="n"/>
       <c r="U104" s="8" t="n"/>
-      <c r="V104" s="8" t="n"/>
     </row>
     <row r="105">
       <c r="D105" s="3" t="n"/>
-      <c r="E105" s="3" t="n"/>
+      <c r="E105" s="8" t="n"/>
       <c r="F105" s="8" t="n"/>
       <c r="G105" s="3" t="n"/>
-      <c r="H105" s="8" t="n"/>
-      <c r="I105" s="3" t="n"/>
+      <c r="H105" s="3" t="n"/>
+      <c r="I105" s="8" t="n"/>
       <c r="J105" s="8" t="n"/>
       <c r="K105" s="8" t="n"/>
-      <c r="L105" s="3" t="n"/>
+      <c r="L105" s="8" t="n"/>
       <c r="M105" s="8" t="n"/>
       <c r="N105" s="8" t="n"/>
       <c r="O105" s="8" t="n"/>
       <c r="P105" s="8" t="n"/>
       <c r="Q105" s="8" t="n"/>
-      <c r="R105" s="8" t="n"/>
+      <c r="R105" s="3" t="n"/>
       <c r="S105" s="3" t="n"/>
-      <c r="T105" s="3" t="n"/>
+      <c r="T105" s="8" t="n"/>
       <c r="U105" s="8" t="n"/>
-      <c r="V105" s="8" t="n"/>
     </row>
     <row r="106">
       <c r="D106" s="3" t="n"/>
-      <c r="E106" s="3" t="n"/>
+      <c r="E106" s="8" t="n"/>
       <c r="F106" s="8" t="n"/>
       <c r="G106" s="3" t="n"/>
-      <c r="H106" s="8" t="n"/>
-      <c r="I106" s="3" t="n"/>
+      <c r="H106" s="3" t="n"/>
+      <c r="I106" s="8" t="n"/>
       <c r="J106" s="8" t="n"/>
       <c r="K106" s="8" t="n"/>
-      <c r="L106" s="3" t="n"/>
+      <c r="L106" s="8" t="n"/>
       <c r="M106" s="8" t="n"/>
       <c r="N106" s="8" t="n"/>
       <c r="O106" s="8" t="n"/>
       <c r="P106" s="8" t="n"/>
       <c r="Q106" s="8" t="n"/>
-      <c r="R106" s="8" t="n"/>
+      <c r="R106" s="3" t="n"/>
       <c r="S106" s="3" t="n"/>
-      <c r="T106" s="3" t="n"/>
+      <c r="T106" s="8" t="n"/>
       <c r="U106" s="8" t="n"/>
-      <c r="V106" s="8" t="n"/>
     </row>
     <row r="107">
       <c r="D107" s="3" t="n"/>
-      <c r="E107" s="3" t="n"/>
+      <c r="E107" s="8" t="n"/>
       <c r="F107" s="8" t="n"/>
       <c r="G107" s="3" t="n"/>
-      <c r="H107" s="8" t="n"/>
-      <c r="I107" s="3" t="n"/>
+      <c r="H107" s="3" t="n"/>
+      <c r="I107" s="8" t="n"/>
       <c r="J107" s="8" t="n"/>
       <c r="K107" s="8" t="n"/>
-      <c r="L107" s="3" t="n"/>
+      <c r="L107" s="8" t="n"/>
       <c r="M107" s="8" t="n"/>
       <c r="N107" s="8" t="n"/>
       <c r="O107" s="8" t="n"/>
       <c r="P107" s="8" t="n"/>
       <c r="Q107" s="8" t="n"/>
-      <c r="R107" s="8" t="n"/>
+      <c r="R107" s="3" t="n"/>
       <c r="S107" s="3" t="n"/>
-      <c r="T107" s="3" t="n"/>
+      <c r="T107" s="8" t="n"/>
       <c r="U107" s="8" t="n"/>
-      <c r="V107" s="8" t="n"/>
     </row>
     <row r="108">
       <c r="D108" s="3" t="n"/>
-      <c r="E108" s="3" t="n"/>
+      <c r="E108" s="8" t="n"/>
       <c r="F108" s="8" t="n"/>
       <c r="G108" s="3" t="n"/>
-      <c r="H108" s="8" t="n"/>
-      <c r="I108" s="3" t="n"/>
+      <c r="H108" s="3" t="n"/>
+      <c r="I108" s="8" t="n"/>
       <c r="J108" s="8" t="n"/>
       <c r="K108" s="8" t="n"/>
-      <c r="L108" s="3" t="n"/>
+      <c r="L108" s="8" t="n"/>
       <c r="M108" s="8" t="n"/>
       <c r="N108" s="8" t="n"/>
       <c r="O108" s="8" t="n"/>
       <c r="P108" s="8" t="n"/>
       <c r="Q108" s="8" t="n"/>
-      <c r="R108" s="8" t="n"/>
+      <c r="R108" s="3" t="n"/>
       <c r="S108" s="3" t="n"/>
-      <c r="T108" s="3" t="n"/>
+      <c r="T108" s="8" t="n"/>
       <c r="U108" s="8" t="n"/>
-      <c r="V108" s="8" t="n"/>
     </row>
     <row r="109">
       <c r="D109" s="3" t="n"/>
-      <c r="E109" s="3" t="n"/>
+      <c r="E109" s="8" t="n"/>
       <c r="F109" s="8" t="n"/>
       <c r="G109" s="3" t="n"/>
-      <c r="H109" s="8" t="n"/>
-      <c r="I109" s="3" t="n"/>
+      <c r="H109" s="3" t="n"/>
+      <c r="I109" s="8" t="n"/>
       <c r="J109" s="8" t="n"/>
       <c r="K109" s="8" t="n"/>
-      <c r="L109" s="3" t="n"/>
+      <c r="L109" s="8" t="n"/>
       <c r="M109" s="8" t="n"/>
       <c r="N109" s="8" t="n"/>
       <c r="O109" s="8" t="n"/>
       <c r="P109" s="8" t="n"/>
       <c r="Q109" s="8" t="n"/>
-      <c r="R109" s="8" t="n"/>
+      <c r="R109" s="3" t="n"/>
       <c r="S109" s="3" t="n"/>
-      <c r="T109" s="3" t="n"/>
+      <c r="T109" s="8" t="n"/>
       <c r="U109" s="8" t="n"/>
-      <c r="V109" s="8" t="n"/>
-    </row>
-    <row r="111" ht="22" customHeight="1">
-      <c r="D111" s="10" t="inlineStr">
-        <is>
-          <t>メッセージ一覧</t>
-        </is>
-      </c>
-      <c r="E111" s="11" t="n"/>
-      <c r="F111" s="11" t="n"/>
-      <c r="G111" s="11" t="n"/>
-      <c r="H111" s="11" t="n"/>
-      <c r="I111" s="11" t="n"/>
-      <c r="J111" s="11" t="n"/>
-      <c r="K111" s="11" t="n"/>
-      <c r="L111" s="11" t="n"/>
-      <c r="M111" s="11" t="n"/>
-      <c r="N111" s="11" t="n"/>
-      <c r="O111" s="11" t="n"/>
-      <c r="P111" s="11" t="n"/>
-      <c r="Q111" s="11" t="n"/>
-      <c r="R111" s="11" t="n"/>
-      <c r="S111" s="11" t="n"/>
-      <c r="T111" s="11" t="n"/>
-      <c r="U111" s="11" t="n"/>
-      <c r="V111" s="11" t="n"/>
-    </row>
-    <row r="112" ht="30" customHeight="1">
-      <c r="D112" s="2" t="inlineStr">
-        <is>
-          <t>メッセージID</t>
-        </is>
-      </c>
-      <c r="E112" s="13" t="n"/>
-      <c r="F112" s="13" t="n"/>
-      <c r="G112" s="2" t="inlineStr">
-        <is>
-          <t>種別</t>
-        </is>
-      </c>
-      <c r="H112" s="2" t="inlineStr">
-        <is>
-          <t>文言（日本語）</t>
-        </is>
-      </c>
-      <c r="I112" s="2" t="inlineStr">
-        <is>
-          <t>文言（ベトナム語）</t>
-        </is>
-      </c>
-      <c r="J112" s="13" t="n"/>
-      <c r="K112" s="13" t="n"/>
-      <c r="L112" s="2" t="inlineStr">
-        <is>
-          <t>文言（英語）</t>
-        </is>
-      </c>
-      <c r="M112" s="13" t="n"/>
-      <c r="N112" s="13" t="n"/>
-      <c r="O112" s="13" t="n"/>
-      <c r="P112" s="13" t="n"/>
-      <c r="Q112" s="13" t="n"/>
-      <c r="R112" s="2" t="inlineStr">
-        <is>
-          <t>表示方法</t>
-        </is>
-      </c>
-      <c r="S112" s="2" t="inlineStr">
-        <is>
-          <t>備考</t>
-        </is>
-      </c>
-      <c r="T112" s="13" t="n"/>
-      <c r="U112" s="13" t="n"/>
-      <c r="V112" s="13" t="n"/>
+    </row>
+    <row r="110">
+      <c r="D110" s="3" t="n"/>
+      <c r="E110" s="8" t="n"/>
+      <c r="F110" s="8" t="n"/>
+      <c r="G110" s="3" t="n"/>
+      <c r="H110" s="3" t="n"/>
+      <c r="I110" s="8" t="n"/>
+      <c r="J110" s="8" t="n"/>
+      <c r="K110" s="8" t="n"/>
+      <c r="L110" s="8" t="n"/>
+      <c r="M110" s="8" t="n"/>
+      <c r="N110" s="8" t="n"/>
+      <c r="O110" s="8" t="n"/>
+      <c r="P110" s="8" t="n"/>
+      <c r="Q110" s="8" t="n"/>
+      <c r="R110" s="3" t="n"/>
+      <c r="S110" s="3" t="n"/>
+      <c r="T110" s="8" t="n"/>
+      <c r="U110" s="8" t="n"/>
+    </row>
+    <row r="111">
+      <c r="D111" s="3" t="n"/>
+      <c r="E111" s="8" t="n"/>
+      <c r="F111" s="8" t="n"/>
+      <c r="G111" s="3" t="n"/>
+      <c r="H111" s="3" t="n"/>
+      <c r="I111" s="8" t="n"/>
+      <c r="J111" s="8" t="n"/>
+      <c r="K111" s="8" t="n"/>
+      <c r="L111" s="8" t="n"/>
+      <c r="M111" s="8" t="n"/>
+      <c r="N111" s="8" t="n"/>
+      <c r="O111" s="8" t="n"/>
+      <c r="P111" s="8" t="n"/>
+      <c r="Q111" s="8" t="n"/>
+      <c r="R111" s="3" t="n"/>
+      <c r="S111" s="3" t="n"/>
+      <c r="T111" s="8" t="n"/>
+      <c r="U111" s="8" t="n"/>
+    </row>
+    <row r="112">
+      <c r="D112" s="3" t="n"/>
+      <c r="E112" s="8" t="n"/>
+      <c r="F112" s="8" t="n"/>
+      <c r="G112" s="3" t="n"/>
+      <c r="H112" s="3" t="n"/>
+      <c r="I112" s="8" t="n"/>
+      <c r="J112" s="8" t="n"/>
+      <c r="K112" s="8" t="n"/>
+      <c r="L112" s="8" t="n"/>
+      <c r="M112" s="8" t="n"/>
+      <c r="N112" s="8" t="n"/>
+      <c r="O112" s="8" t="n"/>
+      <c r="P112" s="8" t="n"/>
+      <c r="Q112" s="8" t="n"/>
+      <c r="R112" s="3" t="n"/>
+      <c r="S112" s="3" t="n"/>
+      <c r="T112" s="8" t="n"/>
+      <c r="U112" s="8" t="n"/>
     </row>
     <row r="113">
       <c r="D113" s="3" t="n"/>
@@ -3258,10 +3124,10 @@
       <c r="F113" s="8" t="n"/>
       <c r="G113" s="3" t="n"/>
       <c r="H113" s="3" t="n"/>
-      <c r="I113" s="3" t="n"/>
+      <c r="I113" s="8" t="n"/>
       <c r="J113" s="8" t="n"/>
       <c r="K113" s="8" t="n"/>
-      <c r="L113" s="3" t="n"/>
+      <c r="L113" s="8" t="n"/>
       <c r="M113" s="8" t="n"/>
       <c r="N113" s="8" t="n"/>
       <c r="O113" s="8" t="n"/>
@@ -3271,7 +3137,6 @@
       <c r="S113" s="3" t="n"/>
       <c r="T113" s="8" t="n"/>
       <c r="U113" s="8" t="n"/>
-      <c r="V113" s="8" t="n"/>
     </row>
     <row r="114">
       <c r="D114" s="3" t="n"/>
@@ -3279,10 +3144,10 @@
       <c r="F114" s="8" t="n"/>
       <c r="G114" s="3" t="n"/>
       <c r="H114" s="3" t="n"/>
-      <c r="I114" s="3" t="n"/>
+      <c r="I114" s="8" t="n"/>
       <c r="J114" s="8" t="n"/>
       <c r="K114" s="8" t="n"/>
-      <c r="L114" s="3" t="n"/>
+      <c r="L114" s="8" t="n"/>
       <c r="M114" s="8" t="n"/>
       <c r="N114" s="8" t="n"/>
       <c r="O114" s="8" t="n"/>
@@ -3292,354 +3157,338 @@
       <c r="S114" s="3" t="n"/>
       <c r="T114" s="8" t="n"/>
       <c r="U114" s="8" t="n"/>
-      <c r="V114" s="8" t="n"/>
-    </row>
-    <row r="115">
-      <c r="D115" s="3" t="n"/>
-      <c r="E115" s="8" t="n"/>
-      <c r="F115" s="8" t="n"/>
-      <c r="G115" s="3" t="n"/>
-      <c r="H115" s="3" t="n"/>
-      <c r="I115" s="3" t="n"/>
-      <c r="J115" s="8" t="n"/>
-      <c r="K115" s="8" t="n"/>
-      <c r="L115" s="3" t="n"/>
-      <c r="M115" s="8" t="n"/>
-      <c r="N115" s="8" t="n"/>
-      <c r="O115" s="8" t="n"/>
-      <c r="P115" s="8" t="n"/>
-      <c r="Q115" s="8" t="n"/>
-      <c r="R115" s="3" t="n"/>
-      <c r="S115" s="3" t="n"/>
-      <c r="T115" s="8" t="n"/>
-      <c r="U115" s="8" t="n"/>
-      <c r="V115" s="8" t="n"/>
-    </row>
-    <row r="116">
-      <c r="D116" s="3" t="n"/>
-      <c r="E116" s="8" t="n"/>
-      <c r="F116" s="8" t="n"/>
-      <c r="G116" s="3" t="n"/>
-      <c r="H116" s="3" t="n"/>
-      <c r="I116" s="3" t="n"/>
-      <c r="J116" s="8" t="n"/>
-      <c r="K116" s="8" t="n"/>
-      <c r="L116" s="3" t="n"/>
-      <c r="M116" s="8" t="n"/>
-      <c r="N116" s="8" t="n"/>
-      <c r="O116" s="8" t="n"/>
-      <c r="P116" s="8" t="n"/>
-      <c r="Q116" s="8" t="n"/>
-      <c r="R116" s="3" t="n"/>
-      <c r="S116" s="3" t="n"/>
-      <c r="T116" s="8" t="n"/>
-      <c r="U116" s="8" t="n"/>
-      <c r="V116" s="8" t="n"/>
-    </row>
-    <row r="117">
-      <c r="D117" s="3" t="n"/>
-      <c r="E117" s="8" t="n"/>
-      <c r="F117" s="8" t="n"/>
-      <c r="G117" s="3" t="n"/>
-      <c r="H117" s="3" t="n"/>
-      <c r="I117" s="3" t="n"/>
-      <c r="J117" s="8" t="n"/>
-      <c r="K117" s="8" t="n"/>
-      <c r="L117" s="3" t="n"/>
-      <c r="M117" s="8" t="n"/>
-      <c r="N117" s="8" t="n"/>
-      <c r="O117" s="8" t="n"/>
-      <c r="P117" s="8" t="n"/>
-      <c r="Q117" s="8" t="n"/>
-      <c r="R117" s="3" t="n"/>
-      <c r="S117" s="3" t="n"/>
-      <c r="T117" s="8" t="n"/>
-      <c r="U117" s="8" t="n"/>
-      <c r="V117" s="8" t="n"/>
+    </row>
+    <row r="116" ht="22" customHeight="1">
+      <c r="D116" s="10" t="inlineStr">
+        <is>
+          <t>未決事項</t>
+        </is>
+      </c>
+      <c r="E116" s="11" t="n"/>
+      <c r="F116" s="11" t="n"/>
+      <c r="G116" s="11" t="n"/>
+      <c r="H116" s="11" t="n"/>
+      <c r="I116" s="11" t="n"/>
+      <c r="J116" s="11" t="n"/>
+      <c r="K116" s="11" t="n"/>
+      <c r="L116" s="11" t="n"/>
+      <c r="M116" s="11" t="n"/>
+      <c r="N116" s="11" t="n"/>
+      <c r="O116" s="11" t="n"/>
+      <c r="P116" s="11" t="n"/>
+      <c r="Q116" s="11" t="n"/>
+      <c r="R116" s="11" t="n"/>
+      <c r="S116" s="11" t="n"/>
+      <c r="T116" s="11" t="n"/>
+      <c r="U116" s="11" t="n"/>
+    </row>
+    <row r="117" ht="30" customHeight="1">
+      <c r="D117" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E117" s="2" t="inlineStr">
+        <is>
+          <t>対象項目No</t>
+        </is>
+      </c>
+      <c r="F117" s="13" t="n"/>
+      <c r="G117" s="2" t="inlineStr">
+        <is>
+          <t>質問</t>
+        </is>
+      </c>
+      <c r="H117" s="13" t="n"/>
+      <c r="I117" s="13" t="n"/>
+      <c r="J117" s="13" t="n"/>
+      <c r="K117" s="2" t="inlineStr">
+        <is>
+          <t>決定内容</t>
+        </is>
+      </c>
+      <c r="L117" s="13" t="n"/>
+      <c r="M117" s="13" t="n"/>
+      <c r="N117" s="13" t="n"/>
+      <c r="O117" s="13" t="n"/>
+      <c r="P117" s="13" t="n"/>
+      <c r="Q117" s="13" t="n"/>
+      <c r="R117" s="13" t="n"/>
+      <c r="S117" s="2" t="inlineStr">
+        <is>
+          <t>決定者</t>
+        </is>
+      </c>
+      <c r="T117" s="2" t="inlineStr">
+        <is>
+          <t>決定日</t>
+        </is>
+      </c>
+      <c r="U117" s="2" t="inlineStr">
+        <is>
+          <t>状態</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="D118" s="3" t="n"/>
-      <c r="E118" s="8" t="n"/>
+      <c r="E118" s="3" t="n"/>
       <c r="F118" s="8" t="n"/>
       <c r="G118" s="3" t="n"/>
-      <c r="H118" s="3" t="n"/>
-      <c r="I118" s="3" t="n"/>
+      <c r="H118" s="8" t="n"/>
+      <c r="I118" s="8" t="n"/>
       <c r="J118" s="8" t="n"/>
-      <c r="K118" s="8" t="n"/>
-      <c r="L118" s="3" t="n"/>
+      <c r="K118" s="3" t="n"/>
+      <c r="L118" s="8" t="n"/>
       <c r="M118" s="8" t="n"/>
       <c r="N118" s="8" t="n"/>
       <c r="O118" s="8" t="n"/>
       <c r="P118" s="8" t="n"/>
       <c r="Q118" s="8" t="n"/>
-      <c r="R118" s="3" t="n"/>
+      <c r="R118" s="8" t="n"/>
       <c r="S118" s="3" t="n"/>
-      <c r="T118" s="8" t="n"/>
-      <c r="U118" s="8" t="n"/>
-      <c r="V118" s="8" t="n"/>
+      <c r="T118" s="4" t="n"/>
+      <c r="U118" s="3" t="n"/>
     </row>
     <row r="119">
       <c r="D119" s="3" t="n"/>
-      <c r="E119" s="8" t="n"/>
+      <c r="E119" s="3" t="n"/>
       <c r="F119" s="8" t="n"/>
       <c r="G119" s="3" t="n"/>
-      <c r="H119" s="3" t="n"/>
-      <c r="I119" s="3" t="n"/>
+      <c r="H119" s="8" t="n"/>
+      <c r="I119" s="8" t="n"/>
       <c r="J119" s="8" t="n"/>
-      <c r="K119" s="8" t="n"/>
-      <c r="L119" s="3" t="n"/>
+      <c r="K119" s="3" t="n"/>
+      <c r="L119" s="8" t="n"/>
       <c r="M119" s="8" t="n"/>
       <c r="N119" s="8" t="n"/>
       <c r="O119" s="8" t="n"/>
       <c r="P119" s="8" t="n"/>
       <c r="Q119" s="8" t="n"/>
-      <c r="R119" s="3" t="n"/>
+      <c r="R119" s="8" t="n"/>
       <c r="S119" s="3" t="n"/>
-      <c r="T119" s="8" t="n"/>
-      <c r="U119" s="8" t="n"/>
-      <c r="V119" s="8" t="n"/>
+      <c r="T119" s="4" t="n"/>
+      <c r="U119" s="3" t="n"/>
     </row>
     <row r="120">
       <c r="D120" s="3" t="n"/>
-      <c r="E120" s="8" t="n"/>
+      <c r="E120" s="3" t="n"/>
       <c r="F120" s="8" t="n"/>
       <c r="G120" s="3" t="n"/>
-      <c r="H120" s="3" t="n"/>
-      <c r="I120" s="3" t="n"/>
+      <c r="H120" s="8" t="n"/>
+      <c r="I120" s="8" t="n"/>
       <c r="J120" s="8" t="n"/>
-      <c r="K120" s="8" t="n"/>
-      <c r="L120" s="3" t="n"/>
+      <c r="K120" s="3" t="n"/>
+      <c r="L120" s="8" t="n"/>
       <c r="M120" s="8" t="n"/>
       <c r="N120" s="8" t="n"/>
       <c r="O120" s="8" t="n"/>
       <c r="P120" s="8" t="n"/>
       <c r="Q120" s="8" t="n"/>
-      <c r="R120" s="3" t="n"/>
+      <c r="R120" s="8" t="n"/>
       <c r="S120" s="3" t="n"/>
-      <c r="T120" s="8" t="n"/>
-      <c r="U120" s="8" t="n"/>
-      <c r="V120" s="8" t="n"/>
+      <c r="T120" s="4" t="n"/>
+      <c r="U120" s="3" t="n"/>
     </row>
     <row r="121">
       <c r="D121" s="3" t="n"/>
-      <c r="E121" s="8" t="n"/>
+      <c r="E121" s="3" t="n"/>
       <c r="F121" s="8" t="n"/>
       <c r="G121" s="3" t="n"/>
-      <c r="H121" s="3" t="n"/>
-      <c r="I121" s="3" t="n"/>
+      <c r="H121" s="8" t="n"/>
+      <c r="I121" s="8" t="n"/>
       <c r="J121" s="8" t="n"/>
-      <c r="K121" s="8" t="n"/>
-      <c r="L121" s="3" t="n"/>
+      <c r="K121" s="3" t="n"/>
+      <c r="L121" s="8" t="n"/>
       <c r="M121" s="8" t="n"/>
       <c r="N121" s="8" t="n"/>
       <c r="O121" s="8" t="n"/>
       <c r="P121" s="8" t="n"/>
       <c r="Q121" s="8" t="n"/>
-      <c r="R121" s="3" t="n"/>
+      <c r="R121" s="8" t="n"/>
       <c r="S121" s="3" t="n"/>
-      <c r="T121" s="8" t="n"/>
-      <c r="U121" s="8" t="n"/>
-      <c r="V121" s="8" t="n"/>
+      <c r="T121" s="4" t="n"/>
+      <c r="U121" s="3" t="n"/>
     </row>
     <row r="122">
       <c r="D122" s="3" t="n"/>
-      <c r="E122" s="8" t="n"/>
+      <c r="E122" s="3" t="n"/>
       <c r="F122" s="8" t="n"/>
       <c r="G122" s="3" t="n"/>
-      <c r="H122" s="3" t="n"/>
-      <c r="I122" s="3" t="n"/>
+      <c r="H122" s="8" t="n"/>
+      <c r="I122" s="8" t="n"/>
       <c r="J122" s="8" t="n"/>
-      <c r="K122" s="8" t="n"/>
-      <c r="L122" s="3" t="n"/>
+      <c r="K122" s="3" t="n"/>
+      <c r="L122" s="8" t="n"/>
       <c r="M122" s="8" t="n"/>
       <c r="N122" s="8" t="n"/>
       <c r="O122" s="8" t="n"/>
       <c r="P122" s="8" t="n"/>
       <c r="Q122" s="8" t="n"/>
-      <c r="R122" s="3" t="n"/>
+      <c r="R122" s="8" t="n"/>
       <c r="S122" s="3" t="n"/>
-      <c r="T122" s="8" t="n"/>
-      <c r="U122" s="8" t="n"/>
-      <c r="V122" s="8" t="n"/>
+      <c r="T122" s="4" t="n"/>
+      <c r="U122" s="3" t="n"/>
     </row>
     <row r="123">
       <c r="D123" s="3" t="n"/>
-      <c r="E123" s="8" t="n"/>
+      <c r="E123" s="3" t="n"/>
       <c r="F123" s="8" t="n"/>
       <c r="G123" s="3" t="n"/>
-      <c r="H123" s="3" t="n"/>
-      <c r="I123" s="3" t="n"/>
+      <c r="H123" s="8" t="n"/>
+      <c r="I123" s="8" t="n"/>
       <c r="J123" s="8" t="n"/>
-      <c r="K123" s="8" t="n"/>
-      <c r="L123" s="3" t="n"/>
+      <c r="K123" s="3" t="n"/>
+      <c r="L123" s="8" t="n"/>
       <c r="M123" s="8" t="n"/>
       <c r="N123" s="8" t="n"/>
       <c r="O123" s="8" t="n"/>
       <c r="P123" s="8" t="n"/>
       <c r="Q123" s="8" t="n"/>
-      <c r="R123" s="3" t="n"/>
+      <c r="R123" s="8" t="n"/>
       <c r="S123" s="3" t="n"/>
-      <c r="T123" s="8" t="n"/>
-      <c r="U123" s="8" t="n"/>
-      <c r="V123" s="8" t="n"/>
+      <c r="T123" s="4" t="n"/>
+      <c r="U123" s="3" t="n"/>
     </row>
     <row r="124">
       <c r="D124" s="3" t="n"/>
-      <c r="E124" s="8" t="n"/>
+      <c r="E124" s="3" t="n"/>
       <c r="F124" s="8" t="n"/>
       <c r="G124" s="3" t="n"/>
-      <c r="H124" s="3" t="n"/>
-      <c r="I124" s="3" t="n"/>
+      <c r="H124" s="8" t="n"/>
+      <c r="I124" s="8" t="n"/>
       <c r="J124" s="8" t="n"/>
-      <c r="K124" s="8" t="n"/>
-      <c r="L124" s="3" t="n"/>
+      <c r="K124" s="3" t="n"/>
+      <c r="L124" s="8" t="n"/>
       <c r="M124" s="8" t="n"/>
       <c r="N124" s="8" t="n"/>
       <c r="O124" s="8" t="n"/>
       <c r="P124" s="8" t="n"/>
       <c r="Q124" s="8" t="n"/>
-      <c r="R124" s="3" t="n"/>
+      <c r="R124" s="8" t="n"/>
       <c r="S124" s="3" t="n"/>
-      <c r="T124" s="8" t="n"/>
-      <c r="U124" s="8" t="n"/>
-      <c r="V124" s="8" t="n"/>
+      <c r="T124" s="4" t="n"/>
+      <c r="U124" s="3" t="n"/>
     </row>
     <row r="125">
       <c r="D125" s="3" t="n"/>
-      <c r="E125" s="8" t="n"/>
+      <c r="E125" s="3" t="n"/>
       <c r="F125" s="8" t="n"/>
       <c r="G125" s="3" t="n"/>
-      <c r="H125" s="3" t="n"/>
-      <c r="I125" s="3" t="n"/>
+      <c r="H125" s="8" t="n"/>
+      <c r="I125" s="8" t="n"/>
       <c r="J125" s="8" t="n"/>
-      <c r="K125" s="8" t="n"/>
-      <c r="L125" s="3" t="n"/>
+      <c r="K125" s="3" t="n"/>
+      <c r="L125" s="8" t="n"/>
       <c r="M125" s="8" t="n"/>
       <c r="N125" s="8" t="n"/>
       <c r="O125" s="8" t="n"/>
       <c r="P125" s="8" t="n"/>
       <c r="Q125" s="8" t="n"/>
-      <c r="R125" s="3" t="n"/>
+      <c r="R125" s="8" t="n"/>
       <c r="S125" s="3" t="n"/>
-      <c r="T125" s="8" t="n"/>
-      <c r="U125" s="8" t="n"/>
-      <c r="V125" s="8" t="n"/>
+      <c r="T125" s="4" t="n"/>
+      <c r="U125" s="3" t="n"/>
     </row>
     <row r="126">
       <c r="D126" s="3" t="n"/>
-      <c r="E126" s="8" t="n"/>
+      <c r="E126" s="3" t="n"/>
       <c r="F126" s="8" t="n"/>
       <c r="G126" s="3" t="n"/>
-      <c r="H126" s="3" t="n"/>
-      <c r="I126" s="3" t="n"/>
+      <c r="H126" s="8" t="n"/>
+      <c r="I126" s="8" t="n"/>
       <c r="J126" s="8" t="n"/>
-      <c r="K126" s="8" t="n"/>
-      <c r="L126" s="3" t="n"/>
+      <c r="K126" s="3" t="n"/>
+      <c r="L126" s="8" t="n"/>
       <c r="M126" s="8" t="n"/>
       <c r="N126" s="8" t="n"/>
       <c r="O126" s="8" t="n"/>
       <c r="P126" s="8" t="n"/>
       <c r="Q126" s="8" t="n"/>
-      <c r="R126" s="3" t="n"/>
+      <c r="R126" s="8" t="n"/>
       <c r="S126" s="3" t="n"/>
-      <c r="T126" s="8" t="n"/>
-      <c r="U126" s="8" t="n"/>
-      <c r="V126" s="8" t="n"/>
+      <c r="T126" s="4" t="n"/>
+      <c r="U126" s="3" t="n"/>
     </row>
     <row r="127">
       <c r="D127" s="3" t="n"/>
-      <c r="E127" s="8" t="n"/>
+      <c r="E127" s="3" t="n"/>
       <c r="F127" s="8" t="n"/>
       <c r="G127" s="3" t="n"/>
-      <c r="H127" s="3" t="n"/>
-      <c r="I127" s="3" t="n"/>
+      <c r="H127" s="8" t="n"/>
+      <c r="I127" s="8" t="n"/>
       <c r="J127" s="8" t="n"/>
-      <c r="K127" s="8" t="n"/>
-      <c r="L127" s="3" t="n"/>
+      <c r="K127" s="3" t="n"/>
+      <c r="L127" s="8" t="n"/>
       <c r="M127" s="8" t="n"/>
       <c r="N127" s="8" t="n"/>
       <c r="O127" s="8" t="n"/>
       <c r="P127" s="8" t="n"/>
       <c r="Q127" s="8" t="n"/>
-      <c r="R127" s="3" t="n"/>
+      <c r="R127" s="8" t="n"/>
       <c r="S127" s="3" t="n"/>
-      <c r="T127" s="8" t="n"/>
-      <c r="U127" s="8" t="n"/>
-      <c r="V127" s="8" t="n"/>
-    </row>
-    <row r="129" ht="22" customHeight="1">
-      <c r="D129" s="10" t="inlineStr">
-        <is>
-          <t>未決事項</t>
-        </is>
-      </c>
-      <c r="E129" s="11" t="n"/>
-      <c r="F129" s="11" t="n"/>
-      <c r="G129" s="11" t="n"/>
-      <c r="H129" s="11" t="n"/>
-      <c r="I129" s="11" t="n"/>
-      <c r="J129" s="11" t="n"/>
-      <c r="K129" s="11" t="n"/>
-      <c r="L129" s="11" t="n"/>
-      <c r="M129" s="11" t="n"/>
-      <c r="N129" s="11" t="n"/>
-      <c r="O129" s="11" t="n"/>
-      <c r="P129" s="11" t="n"/>
-      <c r="Q129" s="11" t="n"/>
-      <c r="R129" s="11" t="n"/>
-      <c r="S129" s="11" t="n"/>
-      <c r="T129" s="11" t="n"/>
-      <c r="U129" s="11" t="n"/>
-      <c r="V129" s="11" t="n"/>
-    </row>
-    <row r="130" ht="30" customHeight="1">
-      <c r="D130" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E130" s="2" t="inlineStr">
-        <is>
-          <t>対象項目No</t>
-        </is>
-      </c>
-      <c r="F130" s="13" t="n"/>
-      <c r="G130" s="2" t="inlineStr">
-        <is>
-          <t>質問</t>
-        </is>
-      </c>
-      <c r="H130" s="13" t="n"/>
-      <c r="I130" s="13" t="n"/>
-      <c r="J130" s="13" t="n"/>
-      <c r="K130" s="2" t="inlineStr">
-        <is>
-          <t>決定内容</t>
-        </is>
-      </c>
-      <c r="L130" s="13" t="n"/>
-      <c r="M130" s="13" t="n"/>
-      <c r="N130" s="13" t="n"/>
-      <c r="O130" s="13" t="n"/>
-      <c r="P130" s="13" t="n"/>
-      <c r="Q130" s="13" t="n"/>
-      <c r="R130" s="13" t="n"/>
-      <c r="S130" s="2" t="inlineStr">
-        <is>
-          <t>決定者</t>
-        </is>
-      </c>
-      <c r="T130" s="2" t="inlineStr">
-        <is>
-          <t>決定日</t>
-        </is>
-      </c>
-      <c r="U130" s="2" t="inlineStr">
-        <is>
-          <t>状態</t>
-        </is>
-      </c>
-      <c r="V130" s="13" t="n"/>
+      <c r="T127" s="4" t="n"/>
+      <c r="U127" s="3" t="n"/>
+    </row>
+    <row r="128">
+      <c r="D128" s="3" t="n"/>
+      <c r="E128" s="3" t="n"/>
+      <c r="F128" s="8" t="n"/>
+      <c r="G128" s="3" t="n"/>
+      <c r="H128" s="8" t="n"/>
+      <c r="I128" s="8" t="n"/>
+      <c r="J128" s="8" t="n"/>
+      <c r="K128" s="3" t="n"/>
+      <c r="L128" s="8" t="n"/>
+      <c r="M128" s="8" t="n"/>
+      <c r="N128" s="8" t="n"/>
+      <c r="O128" s="8" t="n"/>
+      <c r="P128" s="8" t="n"/>
+      <c r="Q128" s="8" t="n"/>
+      <c r="R128" s="8" t="n"/>
+      <c r="S128" s="3" t="n"/>
+      <c r="T128" s="4" t="n"/>
+      <c r="U128" s="3" t="n"/>
+    </row>
+    <row r="129">
+      <c r="D129" s="3" t="n"/>
+      <c r="E129" s="3" t="n"/>
+      <c r="F129" s="8" t="n"/>
+      <c r="G129" s="3" t="n"/>
+      <c r="H129" s="8" t="n"/>
+      <c r="I129" s="8" t="n"/>
+      <c r="J129" s="8" t="n"/>
+      <c r="K129" s="3" t="n"/>
+      <c r="L129" s="8" t="n"/>
+      <c r="M129" s="8" t="n"/>
+      <c r="N129" s="8" t="n"/>
+      <c r="O129" s="8" t="n"/>
+      <c r="P129" s="8" t="n"/>
+      <c r="Q129" s="8" t="n"/>
+      <c r="R129" s="8" t="n"/>
+      <c r="S129" s="3" t="n"/>
+      <c r="T129" s="4" t="n"/>
+      <c r="U129" s="3" t="n"/>
+    </row>
+    <row r="130">
+      <c r="D130" s="3" t="n"/>
+      <c r="E130" s="3" t="n"/>
+      <c r="F130" s="8" t="n"/>
+      <c r="G130" s="3" t="n"/>
+      <c r="H130" s="8" t="n"/>
+      <c r="I130" s="8" t="n"/>
+      <c r="J130" s="8" t="n"/>
+      <c r="K130" s="3" t="n"/>
+      <c r="L130" s="8" t="n"/>
+      <c r="M130" s="8" t="n"/>
+      <c r="N130" s="8" t="n"/>
+      <c r="O130" s="8" t="n"/>
+      <c r="P130" s="8" t="n"/>
+      <c r="Q130" s="8" t="n"/>
+      <c r="R130" s="8" t="n"/>
+      <c r="S130" s="3" t="n"/>
+      <c r="T130" s="4" t="n"/>
+      <c r="U130" s="3" t="n"/>
     </row>
     <row r="131">
       <c r="D131" s="3" t="n"/>
@@ -3660,7 +3509,6 @@
       <c r="S131" s="3" t="n"/>
       <c r="T131" s="4" t="n"/>
       <c r="U131" s="3" t="n"/>
-      <c r="V131" s="8" t="n"/>
     </row>
     <row r="132">
       <c r="D132" s="3" t="n"/>
@@ -3681,645 +3529,273 @@
       <c r="S132" s="3" t="n"/>
       <c r="T132" s="4" t="n"/>
       <c r="U132" s="3" t="n"/>
-      <c r="V132" s="8" t="n"/>
-    </row>
-    <row r="133">
-      <c r="D133" s="3" t="n"/>
-      <c r="E133" s="3" t="n"/>
-      <c r="F133" s="8" t="n"/>
-      <c r="G133" s="3" t="n"/>
-      <c r="H133" s="8" t="n"/>
-      <c r="I133" s="8" t="n"/>
-      <c r="J133" s="8" t="n"/>
-      <c r="K133" s="3" t="n"/>
-      <c r="L133" s="8" t="n"/>
-      <c r="M133" s="8" t="n"/>
-      <c r="N133" s="8" t="n"/>
-      <c r="O133" s="8" t="n"/>
-      <c r="P133" s="8" t="n"/>
-      <c r="Q133" s="8" t="n"/>
-      <c r="R133" s="8" t="n"/>
-      <c r="S133" s="3" t="n"/>
-      <c r="T133" s="4" t="n"/>
-      <c r="U133" s="3" t="n"/>
-      <c r="V133" s="8" t="n"/>
-    </row>
-    <row r="134">
-      <c r="D134" s="3" t="n"/>
-      <c r="E134" s="3" t="n"/>
-      <c r="F134" s="8" t="n"/>
-      <c r="G134" s="3" t="n"/>
-      <c r="H134" s="8" t="n"/>
-      <c r="I134" s="8" t="n"/>
-      <c r="J134" s="8" t="n"/>
-      <c r="K134" s="3" t="n"/>
-      <c r="L134" s="8" t="n"/>
-      <c r="M134" s="8" t="n"/>
-      <c r="N134" s="8" t="n"/>
-      <c r="O134" s="8" t="n"/>
-      <c r="P134" s="8" t="n"/>
-      <c r="Q134" s="8" t="n"/>
-      <c r="R134" s="8" t="n"/>
-      <c r="S134" s="3" t="n"/>
-      <c r="T134" s="4" t="n"/>
-      <c r="U134" s="3" t="n"/>
-      <c r="V134" s="8" t="n"/>
-    </row>
-    <row r="135">
-      <c r="D135" s="3" t="n"/>
-      <c r="E135" s="3" t="n"/>
-      <c r="F135" s="8" t="n"/>
-      <c r="G135" s="3" t="n"/>
-      <c r="H135" s="8" t="n"/>
-      <c r="I135" s="8" t="n"/>
-      <c r="J135" s="8" t="n"/>
-      <c r="K135" s="3" t="n"/>
-      <c r="L135" s="8" t="n"/>
-      <c r="M135" s="8" t="n"/>
-      <c r="N135" s="8" t="n"/>
-      <c r="O135" s="8" t="n"/>
-      <c r="P135" s="8" t="n"/>
-      <c r="Q135" s="8" t="n"/>
-      <c r="R135" s="8" t="n"/>
-      <c r="S135" s="3" t="n"/>
-      <c r="T135" s="4" t="n"/>
-      <c r="U135" s="3" t="n"/>
-      <c r="V135" s="8" t="n"/>
-    </row>
-    <row r="136">
-      <c r="D136" s="3" t="n"/>
-      <c r="E136" s="3" t="n"/>
-      <c r="F136" s="8" t="n"/>
-      <c r="G136" s="3" t="n"/>
-      <c r="H136" s="8" t="n"/>
-      <c r="I136" s="8" t="n"/>
-      <c r="J136" s="8" t="n"/>
-      <c r="K136" s="3" t="n"/>
-      <c r="L136" s="8" t="n"/>
-      <c r="M136" s="8" t="n"/>
-      <c r="N136" s="8" t="n"/>
-      <c r="O136" s="8" t="n"/>
-      <c r="P136" s="8" t="n"/>
-      <c r="Q136" s="8" t="n"/>
-      <c r="R136" s="8" t="n"/>
-      <c r="S136" s="3" t="n"/>
-      <c r="T136" s="4" t="n"/>
-      <c r="U136" s="3" t="n"/>
-      <c r="V136" s="8" t="n"/>
-    </row>
-    <row r="137">
-      <c r="D137" s="3" t="n"/>
-      <c r="E137" s="3" t="n"/>
-      <c r="F137" s="8" t="n"/>
-      <c r="G137" s="3" t="n"/>
-      <c r="H137" s="8" t="n"/>
-      <c r="I137" s="8" t="n"/>
-      <c r="J137" s="8" t="n"/>
-      <c r="K137" s="3" t="n"/>
-      <c r="L137" s="8" t="n"/>
-      <c r="M137" s="8" t="n"/>
-      <c r="N137" s="8" t="n"/>
-      <c r="O137" s="8" t="n"/>
-      <c r="P137" s="8" t="n"/>
-      <c r="Q137" s="8" t="n"/>
-      <c r="R137" s="8" t="n"/>
-      <c r="S137" s="3" t="n"/>
-      <c r="T137" s="4" t="n"/>
-      <c r="U137" s="3" t="n"/>
-      <c r="V137" s="8" t="n"/>
-    </row>
-    <row r="138">
-      <c r="D138" s="3" t="n"/>
-      <c r="E138" s="3" t="n"/>
-      <c r="F138" s="8" t="n"/>
-      <c r="G138" s="3" t="n"/>
-      <c r="H138" s="8" t="n"/>
-      <c r="I138" s="8" t="n"/>
-      <c r="J138" s="8" t="n"/>
-      <c r="K138" s="3" t="n"/>
-      <c r="L138" s="8" t="n"/>
-      <c r="M138" s="8" t="n"/>
-      <c r="N138" s="8" t="n"/>
-      <c r="O138" s="8" t="n"/>
-      <c r="P138" s="8" t="n"/>
-      <c r="Q138" s="8" t="n"/>
-      <c r="R138" s="8" t="n"/>
-      <c r="S138" s="3" t="n"/>
-      <c r="T138" s="4" t="n"/>
-      <c r="U138" s="3" t="n"/>
-      <c r="V138" s="8" t="n"/>
-    </row>
-    <row r="139">
-      <c r="D139" s="3" t="n"/>
-      <c r="E139" s="3" t="n"/>
-      <c r="F139" s="8" t="n"/>
-      <c r="G139" s="3" t="n"/>
-      <c r="H139" s="8" t="n"/>
-      <c r="I139" s="8" t="n"/>
-      <c r="J139" s="8" t="n"/>
-      <c r="K139" s="3" t="n"/>
-      <c r="L139" s="8" t="n"/>
-      <c r="M139" s="8" t="n"/>
-      <c r="N139" s="8" t="n"/>
-      <c r="O139" s="8" t="n"/>
-      <c r="P139" s="8" t="n"/>
-      <c r="Q139" s="8" t="n"/>
-      <c r="R139" s="8" t="n"/>
-      <c r="S139" s="3" t="n"/>
-      <c r="T139" s="4" t="n"/>
-      <c r="U139" s="3" t="n"/>
-      <c r="V139" s="8" t="n"/>
-    </row>
-    <row r="140">
-      <c r="D140" s="3" t="n"/>
-      <c r="E140" s="3" t="n"/>
-      <c r="F140" s="8" t="n"/>
-      <c r="G140" s="3" t="n"/>
-      <c r="H140" s="8" t="n"/>
-      <c r="I140" s="8" t="n"/>
-      <c r="J140" s="8" t="n"/>
-      <c r="K140" s="3" t="n"/>
-      <c r="L140" s="8" t="n"/>
-      <c r="M140" s="8" t="n"/>
-      <c r="N140" s="8" t="n"/>
-      <c r="O140" s="8" t="n"/>
-      <c r="P140" s="8" t="n"/>
-      <c r="Q140" s="8" t="n"/>
-      <c r="R140" s="8" t="n"/>
-      <c r="S140" s="3" t="n"/>
-      <c r="T140" s="4" t="n"/>
-      <c r="U140" s="3" t="n"/>
-      <c r="V140" s="8" t="n"/>
-    </row>
-    <row r="141">
-      <c r="D141" s="3" t="n"/>
-      <c r="E141" s="3" t="n"/>
-      <c r="F141" s="8" t="n"/>
-      <c r="G141" s="3" t="n"/>
-      <c r="H141" s="8" t="n"/>
-      <c r="I141" s="8" t="n"/>
-      <c r="J141" s="8" t="n"/>
-      <c r="K141" s="3" t="n"/>
-      <c r="L141" s="8" t="n"/>
-      <c r="M141" s="8" t="n"/>
-      <c r="N141" s="8" t="n"/>
-      <c r="O141" s="8" t="n"/>
-      <c r="P141" s="8" t="n"/>
-      <c r="Q141" s="8" t="n"/>
-      <c r="R141" s="8" t="n"/>
-      <c r="S141" s="3" t="n"/>
-      <c r="T141" s="4" t="n"/>
-      <c r="U141" s="3" t="n"/>
-      <c r="V141" s="8" t="n"/>
-    </row>
-    <row r="142">
-      <c r="D142" s="3" t="n"/>
-      <c r="E142" s="3" t="n"/>
-      <c r="F142" s="8" t="n"/>
-      <c r="G142" s="3" t="n"/>
-      <c r="H142" s="8" t="n"/>
-      <c r="I142" s="8" t="n"/>
-      <c r="J142" s="8" t="n"/>
-      <c r="K142" s="3" t="n"/>
-      <c r="L142" s="8" t="n"/>
-      <c r="M142" s="8" t="n"/>
-      <c r="N142" s="8" t="n"/>
-      <c r="O142" s="8" t="n"/>
-      <c r="P142" s="8" t="n"/>
-      <c r="Q142" s="8" t="n"/>
-      <c r="R142" s="8" t="n"/>
-      <c r="S142" s="3" t="n"/>
-      <c r="T142" s="4" t="n"/>
-      <c r="U142" s="3" t="n"/>
-      <c r="V142" s="8" t="n"/>
-    </row>
-    <row r="143">
-      <c r="D143" s="3" t="n"/>
-      <c r="E143" s="3" t="n"/>
-      <c r="F143" s="8" t="n"/>
-      <c r="G143" s="3" t="n"/>
-      <c r="H143" s="8" t="n"/>
-      <c r="I143" s="8" t="n"/>
-      <c r="J143" s="8" t="n"/>
-      <c r="K143" s="3" t="n"/>
-      <c r="L143" s="8" t="n"/>
-      <c r="M143" s="8" t="n"/>
-      <c r="N143" s="8" t="n"/>
-      <c r="O143" s="8" t="n"/>
-      <c r="P143" s="8" t="n"/>
-      <c r="Q143" s="8" t="n"/>
-      <c r="R143" s="8" t="n"/>
-      <c r="S143" s="3" t="n"/>
-      <c r="T143" s="4" t="n"/>
-      <c r="U143" s="3" t="n"/>
-      <c r="V143" s="8" t="n"/>
-    </row>
-    <row r="144">
-      <c r="D144" s="3" t="n"/>
-      <c r="E144" s="3" t="n"/>
-      <c r="F144" s="8" t="n"/>
-      <c r="G144" s="3" t="n"/>
-      <c r="H144" s="8" t="n"/>
-      <c r="I144" s="8" t="n"/>
-      <c r="J144" s="8" t="n"/>
-      <c r="K144" s="3" t="n"/>
-      <c r="L144" s="8" t="n"/>
-      <c r="M144" s="8" t="n"/>
-      <c r="N144" s="8" t="n"/>
-      <c r="O144" s="8" t="n"/>
-      <c r="P144" s="8" t="n"/>
-      <c r="Q144" s="8" t="n"/>
-      <c r="R144" s="8" t="n"/>
-      <c r="S144" s="3" t="n"/>
-      <c r="T144" s="4" t="n"/>
-      <c r="U144" s="3" t="n"/>
-      <c r="V144" s="8" t="n"/>
-    </row>
-    <row r="145">
-      <c r="D145" s="3" t="n"/>
-      <c r="E145" s="3" t="n"/>
-      <c r="F145" s="8" t="n"/>
-      <c r="G145" s="3" t="n"/>
-      <c r="H145" s="8" t="n"/>
-      <c r="I145" s="8" t="n"/>
-      <c r="J145" s="8" t="n"/>
-      <c r="K145" s="3" t="n"/>
-      <c r="L145" s="8" t="n"/>
-      <c r="M145" s="8" t="n"/>
-      <c r="N145" s="8" t="n"/>
-      <c r="O145" s="8" t="n"/>
-      <c r="P145" s="8" t="n"/>
-      <c r="Q145" s="8" t="n"/>
-      <c r="R145" s="8" t="n"/>
-      <c r="S145" s="3" t="n"/>
-      <c r="T145" s="4" t="n"/>
-      <c r="U145" s="3" t="n"/>
-      <c r="V145" s="8" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="360">
+  <mergeCells count="262">
+    <mergeCell ref="D6:U6"/>
     <mergeCell ref="D60:E60"/>
-    <mergeCell ref="I125:K125"/>
-    <mergeCell ref="I112:K112"/>
-    <mergeCell ref="D116:F116"/>
-    <mergeCell ref="E142:F142"/>
-    <mergeCell ref="G135:J135"/>
-    <mergeCell ref="G62:R62"/>
-    <mergeCell ref="I127:K127"/>
-    <mergeCell ref="I114:K114"/>
-    <mergeCell ref="U136:V136"/>
-    <mergeCell ref="S79:V79"/>
-    <mergeCell ref="L114:Q114"/>
+    <mergeCell ref="S101:U101"/>
+    <mergeCell ref="K121:R121"/>
+    <mergeCell ref="F68:G68"/>
+    <mergeCell ref="H111:Q111"/>
+    <mergeCell ref="E129:F129"/>
+    <mergeCell ref="I87:K87"/>
+    <mergeCell ref="I96:K96"/>
+    <mergeCell ref="H1:U1"/>
+    <mergeCell ref="K123:R123"/>
+    <mergeCell ref="H69:J69"/>
+    <mergeCell ref="G119:J119"/>
+    <mergeCell ref="H104:Q104"/>
+    <mergeCell ref="E131:F131"/>
+    <mergeCell ref="D77:E77"/>
+    <mergeCell ref="E87:F87"/>
+    <mergeCell ref="D102:F102"/>
+    <mergeCell ref="D2:H2"/>
     <mergeCell ref="H75:J75"/>
-    <mergeCell ref="L93:P93"/>
-    <mergeCell ref="E137:F137"/>
+    <mergeCell ref="F80:G80"/>
+    <mergeCell ref="E128:F128"/>
+    <mergeCell ref="H106:Q106"/>
+    <mergeCell ref="K76:U76"/>
+    <mergeCell ref="D61:E61"/>
+    <mergeCell ref="I88:K88"/>
     <mergeCell ref="D70:E70"/>
-    <mergeCell ref="S81:V81"/>
+    <mergeCell ref="G55:U55"/>
     <mergeCell ref="F70:G70"/>
-    <mergeCell ref="L107:R107"/>
-    <mergeCell ref="Q95:V95"/>
-    <mergeCell ref="U131:V131"/>
+    <mergeCell ref="F79:G79"/>
+    <mergeCell ref="G64:U64"/>
     <mergeCell ref="L4:M4"/>
+    <mergeCell ref="D72:E72"/>
     <mergeCell ref="D78:E78"/>
+    <mergeCell ref="S114:U114"/>
+    <mergeCell ref="F72:G72"/>
+    <mergeCell ref="G54:U54"/>
+    <mergeCell ref="F81:G81"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D62:E62"/>
+    <mergeCell ref="D56:E56"/>
     <mergeCell ref="D71:E71"/>
+    <mergeCell ref="E119:F119"/>
     <mergeCell ref="F71:G71"/>
-    <mergeCell ref="D119:F119"/>
+    <mergeCell ref="H78:J78"/>
+    <mergeCell ref="L93:R93"/>
+    <mergeCell ref="S105:U105"/>
+    <mergeCell ref="G56:U56"/>
+    <mergeCell ref="G128:J128"/>
+    <mergeCell ref="E91:F91"/>
+    <mergeCell ref="G91:H91"/>
+    <mergeCell ref="T96:U96"/>
+    <mergeCell ref="D64:E64"/>
+    <mergeCell ref="T90:U90"/>
     <mergeCell ref="D73:E73"/>
-    <mergeCell ref="I113:K113"/>
-    <mergeCell ref="I100:K100"/>
-    <mergeCell ref="I115:K115"/>
-    <mergeCell ref="I102:K102"/>
+    <mergeCell ref="L92:R92"/>
+    <mergeCell ref="D51:E51"/>
+    <mergeCell ref="G94:H94"/>
+    <mergeCell ref="G121:J121"/>
+    <mergeCell ref="E93:F93"/>
+    <mergeCell ref="D105:F105"/>
+    <mergeCell ref="K128:R128"/>
+    <mergeCell ref="H99:Q99"/>
+    <mergeCell ref="H73:J73"/>
+    <mergeCell ref="L94:R94"/>
+    <mergeCell ref="G123:J123"/>
+    <mergeCell ref="K78:U78"/>
+    <mergeCell ref="E117:F117"/>
+    <mergeCell ref="G86:H86"/>
+    <mergeCell ref="T91:U91"/>
+    <mergeCell ref="G57:U57"/>
+    <mergeCell ref="D107:F107"/>
+    <mergeCell ref="E122:F122"/>
     <mergeCell ref="B1:G1"/>
-    <mergeCell ref="L127:Q127"/>
-    <mergeCell ref="S76:V76"/>
-    <mergeCell ref="D85:V85"/>
-    <mergeCell ref="G64:R64"/>
-    <mergeCell ref="D117:F117"/>
-    <mergeCell ref="L103:R103"/>
+    <mergeCell ref="H101:Q101"/>
+    <mergeCell ref="G53:U53"/>
+    <mergeCell ref="E127:F127"/>
+    <mergeCell ref="K80:U80"/>
+    <mergeCell ref="F74:G74"/>
+    <mergeCell ref="I92:K92"/>
+    <mergeCell ref="S103:U103"/>
+    <mergeCell ref="T93:U93"/>
+    <mergeCell ref="F83:G83"/>
+    <mergeCell ref="K79:U79"/>
+    <mergeCell ref="D106:F106"/>
+    <mergeCell ref="K129:R129"/>
+    <mergeCell ref="G58:U58"/>
+    <mergeCell ref="D76:E76"/>
+    <mergeCell ref="L95:R95"/>
+    <mergeCell ref="F76:G76"/>
+    <mergeCell ref="K72:U72"/>
+    <mergeCell ref="K81:U81"/>
+    <mergeCell ref="S108:U108"/>
+    <mergeCell ref="T92:U92"/>
+    <mergeCell ref="H103:Q103"/>
+    <mergeCell ref="D75:E75"/>
+    <mergeCell ref="H77:J77"/>
     <mergeCell ref="D53:E53"/>
-    <mergeCell ref="G51:R51"/>
-    <mergeCell ref="K75:R75"/>
-    <mergeCell ref="H1:V1"/>
-    <mergeCell ref="U137:V137"/>
+    <mergeCell ref="F75:G75"/>
+    <mergeCell ref="H112:Q112"/>
+    <mergeCell ref="S104:U104"/>
+    <mergeCell ref="K131:R131"/>
+    <mergeCell ref="E90:F90"/>
+    <mergeCell ref="D110:F110"/>
+    <mergeCell ref="L87:R87"/>
+    <mergeCell ref="T94:U94"/>
+    <mergeCell ref="K130:R130"/>
+    <mergeCell ref="D98:U98"/>
+    <mergeCell ref="G125:J125"/>
+    <mergeCell ref="K117:R117"/>
+    <mergeCell ref="H114:Q114"/>
+    <mergeCell ref="S106:U106"/>
+    <mergeCell ref="D100:F100"/>
+    <mergeCell ref="G88:H88"/>
+    <mergeCell ref="I90:K90"/>
+    <mergeCell ref="D109:F109"/>
+    <mergeCell ref="E124:F124"/>
+    <mergeCell ref="L89:R89"/>
+    <mergeCell ref="E120:F120"/>
+    <mergeCell ref="K132:R132"/>
+    <mergeCell ref="G127:J127"/>
+    <mergeCell ref="K82:U82"/>
+    <mergeCell ref="H108:Q108"/>
+    <mergeCell ref="T86:U86"/>
+    <mergeCell ref="L88:R88"/>
+    <mergeCell ref="G90:H90"/>
+    <mergeCell ref="T95:U95"/>
+    <mergeCell ref="D111:F111"/>
+    <mergeCell ref="K125:R125"/>
+    <mergeCell ref="D108:F108"/>
     <mergeCell ref="D79:E79"/>
-    <mergeCell ref="L121:Q121"/>
+    <mergeCell ref="I91:K91"/>
     <mergeCell ref="F73:G73"/>
+    <mergeCell ref="D104:F104"/>
+    <mergeCell ref="S107:U107"/>
+    <mergeCell ref="K118:R118"/>
+    <mergeCell ref="K74:U74"/>
+    <mergeCell ref="K69:U69"/>
+    <mergeCell ref="E121:F121"/>
+    <mergeCell ref="K127:R127"/>
+    <mergeCell ref="K83:U83"/>
+    <mergeCell ref="D49:U49"/>
+    <mergeCell ref="D63:E63"/>
+    <mergeCell ref="E130:F130"/>
+    <mergeCell ref="H79:J79"/>
     <mergeCell ref="D81:E81"/>
+    <mergeCell ref="G62:U62"/>
+    <mergeCell ref="I93:K93"/>
+    <mergeCell ref="G129:J129"/>
+    <mergeCell ref="H70:J70"/>
+    <mergeCell ref="D116:U116"/>
+    <mergeCell ref="E123:F123"/>
+    <mergeCell ref="E92:F92"/>
+    <mergeCell ref="D65:E65"/>
+    <mergeCell ref="E132:F132"/>
+    <mergeCell ref="H107:Q107"/>
+    <mergeCell ref="H81:J81"/>
+    <mergeCell ref="S99:U99"/>
+    <mergeCell ref="D52:E52"/>
     <mergeCell ref="G131:J131"/>
-    <mergeCell ref="G58:R58"/>
-    <mergeCell ref="S113:V113"/>
-    <mergeCell ref="D122:F122"/>
-    <mergeCell ref="I123:K123"/>
-    <mergeCell ref="K134:R134"/>
-    <mergeCell ref="S115:V115"/>
+    <mergeCell ref="G124:J124"/>
+    <mergeCell ref="E94:F94"/>
+    <mergeCell ref="L86:R86"/>
+    <mergeCell ref="L2:U2"/>
+    <mergeCell ref="G130:J130"/>
+    <mergeCell ref="O4:P4"/>
+    <mergeCell ref="G117:J117"/>
+    <mergeCell ref="E118:F118"/>
+    <mergeCell ref="G87:H87"/>
     <mergeCell ref="H71:J71"/>
-    <mergeCell ref="E133:F133"/>
-    <mergeCell ref="E108:F108"/>
-    <mergeCell ref="S77:V77"/>
-    <mergeCell ref="S52:V52"/>
-    <mergeCell ref="Q91:V91"/>
+    <mergeCell ref="I94:K94"/>
+    <mergeCell ref="D113:F113"/>
+    <mergeCell ref="H102:Q102"/>
+    <mergeCell ref="H76:J76"/>
+    <mergeCell ref="G126:J126"/>
+    <mergeCell ref="G132:J132"/>
+    <mergeCell ref="E86:F86"/>
+    <mergeCell ref="D67:U67"/>
+    <mergeCell ref="H113:Q113"/>
+    <mergeCell ref="G122:J122"/>
+    <mergeCell ref="E95:F95"/>
+    <mergeCell ref="E89:F89"/>
+    <mergeCell ref="G60:U60"/>
+    <mergeCell ref="D85:U85"/>
+    <mergeCell ref="G89:H89"/>
+    <mergeCell ref="G95:H95"/>
+    <mergeCell ref="K120:R120"/>
+    <mergeCell ref="K71:U71"/>
+    <mergeCell ref="H82:J82"/>
+    <mergeCell ref="S110:U110"/>
+    <mergeCell ref="I86:K86"/>
+    <mergeCell ref="D83:E83"/>
+    <mergeCell ref="F77:G77"/>
+    <mergeCell ref="G59:U59"/>
+    <mergeCell ref="I95:K95"/>
     <mergeCell ref="D55:E55"/>
-    <mergeCell ref="G142:J142"/>
+    <mergeCell ref="I89:K89"/>
+    <mergeCell ref="D99:F99"/>
+    <mergeCell ref="E125:F125"/>
+    <mergeCell ref="G118:J118"/>
+    <mergeCell ref="K73:U73"/>
+    <mergeCell ref="D54:E54"/>
+    <mergeCell ref="G61:U61"/>
+    <mergeCell ref="D101:F101"/>
+    <mergeCell ref="E96:F96"/>
+    <mergeCell ref="G96:H96"/>
+    <mergeCell ref="S111:U111"/>
     <mergeCell ref="D69:E69"/>
     <mergeCell ref="B7:B47"/>
     <mergeCell ref="F69:G69"/>
-    <mergeCell ref="G144:J144"/>
-    <mergeCell ref="S63:V63"/>
-    <mergeCell ref="T104:V104"/>
-    <mergeCell ref="L123:Q123"/>
+    <mergeCell ref="F78:G78"/>
+    <mergeCell ref="K68:U68"/>
+    <mergeCell ref="L96:R96"/>
+    <mergeCell ref="L90:R90"/>
+    <mergeCell ref="H105:Q105"/>
+    <mergeCell ref="D80:E80"/>
+    <mergeCell ref="E88:F88"/>
+    <mergeCell ref="E126:F126"/>
+    <mergeCell ref="D103:F103"/>
+    <mergeCell ref="S112:U112"/>
+    <mergeCell ref="T87:U87"/>
+    <mergeCell ref="D112:F112"/>
+    <mergeCell ref="K126:R126"/>
     <mergeCell ref="H72:J72"/>
-    <mergeCell ref="D86:H86"/>
-    <mergeCell ref="S126:V126"/>
-    <mergeCell ref="L124:Q124"/>
-    <mergeCell ref="S121:V121"/>
-    <mergeCell ref="K71:R71"/>
-    <mergeCell ref="I124:K124"/>
-    <mergeCell ref="K73:R73"/>
-    <mergeCell ref="D82:E82"/>
-    <mergeCell ref="F82:G82"/>
-    <mergeCell ref="S116:V116"/>
-    <mergeCell ref="I126:K126"/>
-    <mergeCell ref="K137:R137"/>
-    <mergeCell ref="E109:F109"/>
-    <mergeCell ref="H83:J83"/>
-    <mergeCell ref="E145:F145"/>
-    <mergeCell ref="S118:V118"/>
-    <mergeCell ref="E139:F139"/>
-    <mergeCell ref="K74:R74"/>
-    <mergeCell ref="K68:R68"/>
-    <mergeCell ref="K139:R139"/>
-    <mergeCell ref="D77:E77"/>
-    <mergeCell ref="T100:V100"/>
-    <mergeCell ref="G145:J145"/>
-    <mergeCell ref="S71:V71"/>
-    <mergeCell ref="D72:E72"/>
-    <mergeCell ref="S58:V58"/>
-    <mergeCell ref="F72:G72"/>
-    <mergeCell ref="G108:H108"/>
-    <mergeCell ref="S73:V73"/>
-    <mergeCell ref="H78:J78"/>
-    <mergeCell ref="Q87:V87"/>
-    <mergeCell ref="D92:H92"/>
-    <mergeCell ref="D49:V49"/>
-    <mergeCell ref="S112:V112"/>
-    <mergeCell ref="D94:H94"/>
-    <mergeCell ref="H73:J73"/>
-    <mergeCell ref="Q93:V93"/>
-    <mergeCell ref="S124:V124"/>
-    <mergeCell ref="F83:G83"/>
-    <mergeCell ref="K138:R138"/>
-    <mergeCell ref="K76:R76"/>
-    <mergeCell ref="S59:V59"/>
-    <mergeCell ref="S119:V119"/>
-    <mergeCell ref="K140:R140"/>
-    <mergeCell ref="G54:R54"/>
-    <mergeCell ref="S61:V61"/>
-    <mergeCell ref="T102:V102"/>
-    <mergeCell ref="E104:F104"/>
-    <mergeCell ref="G104:H104"/>
-    <mergeCell ref="K77:R77"/>
-    <mergeCell ref="G56:R56"/>
-    <mergeCell ref="I105:K105"/>
-    <mergeCell ref="T103:V103"/>
-    <mergeCell ref="I120:K120"/>
-    <mergeCell ref="G99:H99"/>
-    <mergeCell ref="I101:K101"/>
-    <mergeCell ref="L86:P86"/>
-    <mergeCell ref="E130:F130"/>
-    <mergeCell ref="D63:E63"/>
-    <mergeCell ref="S74:V74"/>
-    <mergeCell ref="H79:J79"/>
-    <mergeCell ref="L100:R100"/>
-    <mergeCell ref="Q88:V88"/>
-    <mergeCell ref="H70:J70"/>
-    <mergeCell ref="E141:F141"/>
-    <mergeCell ref="S114:V114"/>
-    <mergeCell ref="E135:F135"/>
-    <mergeCell ref="E132:F132"/>
-    <mergeCell ref="H81:J81"/>
-    <mergeCell ref="E107:F107"/>
-    <mergeCell ref="D52:E52"/>
-    <mergeCell ref="S51:V51"/>
-    <mergeCell ref="Q90:V90"/>
-    <mergeCell ref="D95:H95"/>
-    <mergeCell ref="G101:H101"/>
-    <mergeCell ref="E143:F143"/>
-    <mergeCell ref="L108:R108"/>
-    <mergeCell ref="K72:R72"/>
-    <mergeCell ref="H76:J76"/>
-    <mergeCell ref="U134:V134"/>
-    <mergeCell ref="U142:V142"/>
-    <mergeCell ref="I108:K108"/>
-    <mergeCell ref="L120:Q120"/>
-    <mergeCell ref="S69:V69"/>
-    <mergeCell ref="K141:R141"/>
-    <mergeCell ref="G106:H106"/>
-    <mergeCell ref="G105:H105"/>
-    <mergeCell ref="S127:V127"/>
-    <mergeCell ref="K83:R83"/>
-    <mergeCell ref="K143:R143"/>
-    <mergeCell ref="G57:R57"/>
-    <mergeCell ref="S64:V64"/>
-    <mergeCell ref="G107:H107"/>
-    <mergeCell ref="L126:Q126"/>
-    <mergeCell ref="G134:J134"/>
-    <mergeCell ref="I121:K121"/>
-    <mergeCell ref="D125:F125"/>
-    <mergeCell ref="D98:V98"/>
-    <mergeCell ref="D112:F112"/>
-    <mergeCell ref="E138:F138"/>
-    <mergeCell ref="L113:Q113"/>
-    <mergeCell ref="D127:F127"/>
+    <mergeCell ref="D57:E57"/>
+    <mergeCell ref="H80:J80"/>
+    <mergeCell ref="K122:R122"/>
+    <mergeCell ref="K119:R119"/>
+    <mergeCell ref="G65:U65"/>
+    <mergeCell ref="T89:U89"/>
+    <mergeCell ref="L91:R91"/>
+    <mergeCell ref="G93:H93"/>
     <mergeCell ref="D114:F114"/>
-    <mergeCell ref="L92:P92"/>
-    <mergeCell ref="L115:Q115"/>
-    <mergeCell ref="U130:V130"/>
-    <mergeCell ref="L94:P94"/>
-    <mergeCell ref="S82:V82"/>
+    <mergeCell ref="G120:J120"/>
+    <mergeCell ref="K75:U75"/>
+    <mergeCell ref="G51:U51"/>
+    <mergeCell ref="D3:U3"/>
+    <mergeCell ref="T88:U88"/>
+    <mergeCell ref="G92:H92"/>
+    <mergeCell ref="G63:U63"/>
+    <mergeCell ref="K77:U77"/>
+    <mergeCell ref="G50:U50"/>
+    <mergeCell ref="S113:U113"/>
+    <mergeCell ref="S100:U100"/>
+    <mergeCell ref="D58:E58"/>
+    <mergeCell ref="S109:U109"/>
+    <mergeCell ref="K70:U70"/>
+    <mergeCell ref="G52:U52"/>
     <mergeCell ref="D74:E74"/>
     <mergeCell ref="D68:E68"/>
-    <mergeCell ref="L109:R109"/>
+    <mergeCell ref="H110:Q110"/>
+    <mergeCell ref="D82:E82"/>
+    <mergeCell ref="S102:U102"/>
+    <mergeCell ref="F82:G82"/>
+    <mergeCell ref="H100:Q100"/>
+    <mergeCell ref="H74:J74"/>
+    <mergeCell ref="D50:E50"/>
+    <mergeCell ref="H109:Q109"/>
+    <mergeCell ref="H68:J68"/>
+    <mergeCell ref="H83:J83"/>
     <mergeCell ref="D59:E59"/>
-    <mergeCell ref="U144:V144"/>
-    <mergeCell ref="I103:K103"/>
-    <mergeCell ref="U145:V145"/>
-    <mergeCell ref="U139:V139"/>
-    <mergeCell ref="D129:V129"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="G65:R65"/>
-    <mergeCell ref="D61:E61"/>
-    <mergeCell ref="S72:V72"/>
-    <mergeCell ref="Q86:V86"/>
-    <mergeCell ref="G63:R63"/>
-    <mergeCell ref="G50:R50"/>
-    <mergeCell ref="D62:E62"/>
-    <mergeCell ref="G60:R60"/>
-    <mergeCell ref="L106:R106"/>
-    <mergeCell ref="D56:E56"/>
-    <mergeCell ref="G52:R52"/>
-    <mergeCell ref="G137:J137"/>
-    <mergeCell ref="D64:E64"/>
-    <mergeCell ref="D51:E51"/>
-    <mergeCell ref="I116:K116"/>
-    <mergeCell ref="U138:V138"/>
-    <mergeCell ref="U132:V132"/>
-    <mergeCell ref="G139:J139"/>
-    <mergeCell ref="L116:Q116"/>
-    <mergeCell ref="L95:P95"/>
-    <mergeCell ref="S83:V83"/>
-    <mergeCell ref="L118:Q118"/>
-    <mergeCell ref="L2:V2"/>
-    <mergeCell ref="D3:V3"/>
-    <mergeCell ref="G143:J143"/>
-    <mergeCell ref="L117:Q117"/>
-    <mergeCell ref="D67:V67"/>
-    <mergeCell ref="I118:K118"/>
-    <mergeCell ref="L122:Q122"/>
-    <mergeCell ref="L119:Q119"/>
-    <mergeCell ref="G55:R55"/>
-    <mergeCell ref="D75:E75"/>
-    <mergeCell ref="F75:G75"/>
-    <mergeCell ref="I119:K119"/>
-    <mergeCell ref="K130:R130"/>
-    <mergeCell ref="K132:R132"/>
-    <mergeCell ref="G53:R53"/>
-    <mergeCell ref="G138:J138"/>
-    <mergeCell ref="D65:E65"/>
-    <mergeCell ref="I117:K117"/>
-    <mergeCell ref="G140:J140"/>
-    <mergeCell ref="U141:V141"/>
-    <mergeCell ref="U135:V135"/>
-    <mergeCell ref="O4:P4"/>
-    <mergeCell ref="D87:H87"/>
-    <mergeCell ref="U143:V143"/>
-    <mergeCell ref="S122:V122"/>
-    <mergeCell ref="D6:V6"/>
-    <mergeCell ref="H82:J82"/>
-    <mergeCell ref="E144:F144"/>
-    <mergeCell ref="D83:E83"/>
-    <mergeCell ref="L112:Q112"/>
-    <mergeCell ref="D124:F124"/>
-    <mergeCell ref="K69:R69"/>
-    <mergeCell ref="F78:G78"/>
-    <mergeCell ref="E106:F106"/>
-    <mergeCell ref="I122:K122"/>
-    <mergeCell ref="D126:F126"/>
-    <mergeCell ref="K133:R133"/>
-    <mergeCell ref="D80:E80"/>
-    <mergeCell ref="S54:V54"/>
-    <mergeCell ref="I107:K107"/>
-    <mergeCell ref="K135:R135"/>
-    <mergeCell ref="S56:V56"/>
-    <mergeCell ref="S117:V117"/>
-    <mergeCell ref="D58:E58"/>
-    <mergeCell ref="Q96:V96"/>
-    <mergeCell ref="G141:J141"/>
-    <mergeCell ref="K82:R82"/>
-    <mergeCell ref="D89:H89"/>
-    <mergeCell ref="H74:J74"/>
-    <mergeCell ref="H68:J68"/>
-    <mergeCell ref="D88:H88"/>
-    <mergeCell ref="T108:V108"/>
-    <mergeCell ref="F68:G68"/>
-    <mergeCell ref="D90:H90"/>
-    <mergeCell ref="H69:J69"/>
-    <mergeCell ref="E131:F131"/>
-    <mergeCell ref="T109:V109"/>
-    <mergeCell ref="F80:G80"/>
-    <mergeCell ref="S125:V125"/>
-    <mergeCell ref="F79:G79"/>
-    <mergeCell ref="G136:J136"/>
-    <mergeCell ref="S62:V62"/>
-    <mergeCell ref="E105:F105"/>
-    <mergeCell ref="E99:F99"/>
-    <mergeCell ref="F81:G81"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="S120:V120"/>
-    <mergeCell ref="E101:F101"/>
-    <mergeCell ref="K136:R136"/>
-    <mergeCell ref="K70:R70"/>
-    <mergeCell ref="S57:V57"/>
-    <mergeCell ref="E100:F100"/>
-    <mergeCell ref="G100:H100"/>
-    <mergeCell ref="E136:F136"/>
-    <mergeCell ref="E102:F102"/>
-    <mergeCell ref="G102:H102"/>
-    <mergeCell ref="T106:V106"/>
-    <mergeCell ref="D120:F120"/>
-    <mergeCell ref="F74:G74"/>
-    <mergeCell ref="D96:H96"/>
-    <mergeCell ref="L87:P87"/>
-    <mergeCell ref="S75:V75"/>
-    <mergeCell ref="D76:E76"/>
-    <mergeCell ref="F76:G76"/>
-    <mergeCell ref="L89:P89"/>
-    <mergeCell ref="K131:R131"/>
-    <mergeCell ref="H77:J77"/>
-    <mergeCell ref="L88:P88"/>
-    <mergeCell ref="D91:H91"/>
-    <mergeCell ref="S70:V70"/>
-    <mergeCell ref="D111:V111"/>
-    <mergeCell ref="D93:H93"/>
-    <mergeCell ref="K78:R78"/>
-    <mergeCell ref="S65:V65"/>
-    <mergeCell ref="K142:R142"/>
-    <mergeCell ref="K80:R80"/>
-    <mergeCell ref="S123:V123"/>
-    <mergeCell ref="S50:V50"/>
-    <mergeCell ref="K79:R79"/>
-    <mergeCell ref="K144:R144"/>
-    <mergeCell ref="S60:V60"/>
-    <mergeCell ref="E103:F103"/>
-    <mergeCell ref="G103:H103"/>
-    <mergeCell ref="K81:R81"/>
-    <mergeCell ref="G130:J130"/>
-    <mergeCell ref="D121:F121"/>
-    <mergeCell ref="T105:V105"/>
-    <mergeCell ref="L101:R101"/>
-    <mergeCell ref="T99:V99"/>
-    <mergeCell ref="I109:K109"/>
-    <mergeCell ref="D113:F113"/>
-    <mergeCell ref="G132:J132"/>
-    <mergeCell ref="D123:F123"/>
-    <mergeCell ref="T107:V107"/>
-    <mergeCell ref="T101:V101"/>
-    <mergeCell ref="D115:F115"/>
-    <mergeCell ref="F77:G77"/>
-    <mergeCell ref="L96:P96"/>
-    <mergeCell ref="I104:K104"/>
-    <mergeCell ref="L90:P90"/>
-    <mergeCell ref="E134:F134"/>
-    <mergeCell ref="S78:V78"/>
-    <mergeCell ref="L104:R104"/>
-    <mergeCell ref="D54:E54"/>
-    <mergeCell ref="S53:V53"/>
-    <mergeCell ref="Q92:V92"/>
-    <mergeCell ref="I106:K106"/>
-    <mergeCell ref="S80:V80"/>
-    <mergeCell ref="L91:P91"/>
-    <mergeCell ref="S55:V55"/>
-    <mergeCell ref="Q94:V94"/>
-    <mergeCell ref="L105:R105"/>
-    <mergeCell ref="L99:R99"/>
-    <mergeCell ref="U140:V140"/>
-    <mergeCell ref="E140:F140"/>
-    <mergeCell ref="D57:E57"/>
-    <mergeCell ref="H80:J80"/>
-    <mergeCell ref="D118:F118"/>
-    <mergeCell ref="Q89:V89"/>
-    <mergeCell ref="I99:K99"/>
-    <mergeCell ref="K145:R145"/>
-    <mergeCell ref="G59:R59"/>
-    <mergeCell ref="G109:H109"/>
-    <mergeCell ref="U133:V133"/>
-    <mergeCell ref="L125:Q125"/>
-    <mergeCell ref="L102:R102"/>
-    <mergeCell ref="G61:R61"/>
-    <mergeCell ref="S68:V68"/>
-    <mergeCell ref="D50:E50"/>
-    <mergeCell ref="G133:J133"/>
+    <mergeCell ref="K124:R124"/>
   </mergeCells>
-  <dataValidations count="13">
+  <dataValidations count="10">
     <dataValidation sqref="J2" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"作成中,確定"</formula1>
     </dataValidation>
@@ -4341,22 +3817,13 @@
     <dataValidation sqref="P8:P47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation sqref="J87:J96" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"○,×,表示のみ"</formula1>
-    </dataValidation>
-    <dataValidation sqref="K87:K96" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"○,×,表示のみ"</formula1>
-    </dataValidation>
-    <dataValidation sqref="L87:L96" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"○,×,表示のみ"</formula1>
-    </dataValidation>
-    <dataValidation sqref="G113:G127" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="G100:G114" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"エラー,警告,情報,確認,完了"</formula1>
     </dataValidation>
-    <dataValidation sqref="R113:R127" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="R100:R114" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"インライン,トースト,モーダル,バナー,アラート"</formula1>
     </dataValidation>
-    <dataValidation sqref="U131:U145" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="U118:U132" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"未回答,回答済み"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>